<commit_message>
Ajoute la carte En formation IFMIA - non diplomes (nouveau tableau propre dans Excel)
</commit_message>
<xml_diff>
--- a/suivi.xlsx
+++ b/suivi.xlsx
@@ -3551,13 +3551,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A4:H25"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="20.42578125" bestFit="1" customWidth="1" min="3" max="3"/>
     <col width="20.5703125" bestFit="1" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
     <row r="4">
       <c r="B4" s="31" t="inlineStr">
         <is>
@@ -3566,17 +3569,13 @@
       </c>
       <c r="F4" s="31" t="inlineStr">
         <is>
-          <t>Des arrivees Non diplomés</t>
+          <t>Des arrivees Non diplomes</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="F5" s="14" t="n"/>
-      <c r="G5" s="10" t="inlineStr">
-        <is>
-          <t>Prévue 07/08</t>
-        </is>
-      </c>
+      <c r="G5" s="10" t="n"/>
       <c r="H5" s="14" t="n"/>
     </row>
     <row r="6">
@@ -3602,13 +3601,24 @@
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>FER</t>
-        </is>
-      </c>
-      <c r="G6" s="14" t="n">
-        <v>42</v>
-      </c>
-      <c r="H6" s="14" t="n"/>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>Effectifs</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>Date Integration IFMIA</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Date Integration Usine</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -3641,11 +3651,7 @@
       <c r="D8" s="12" t="n">
         <v>46246</v>
       </c>
-      <c r="F8" s="30" t="inlineStr">
-        <is>
-          <t>Des Arrivees IFMIA Prevue le 11/08</t>
-        </is>
-      </c>
+      <c r="F8" s="30" t="n"/>
       <c r="G8" s="30" t="n"/>
       <c r="H8" s="30" t="n"/>
     </row>
@@ -3664,22 +3670,28 @@
       <c r="D9" s="12" t="n">
         <v>46253</v>
       </c>
-      <c r="F9" s="41" t="n">
-        <v>140</v>
-      </c>
-      <c r="G9" s="55" t="n"/>
-      <c r="H9" s="54" t="n"/>
-    </row>
-    <row r="25">
-      <c r="G25" t="n">
-        <v>612154538</v>
-      </c>
-    </row>
+      <c r="F9" s="41" t="n"/>
+    </row>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="B4:D4"/>
-    <mergeCell ref="F4:H4"/>
-    <mergeCell ref="F9:H9"/>
+    <mergeCell ref="F4:I4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Cartes formation IFMIA en valeurs statiques + popup de bienvenue
</commit_message>
<xml_diff>
--- a/suivi.xlsx
+++ b/suivi.xlsx
@@ -7,11 +7,8 @@
   </bookViews>
   <sheets>
     <sheet name="integration Usine" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Feuil3" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Feuil2" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Feuil1" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="En formation IFMIA" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Indicateurs Manuels" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="En formation IFMIA" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Indicateurs Hebdomadaires" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'integration Usine'!$B$1:$E$105</definedName>
@@ -3028,451 +3025,128 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A4:I9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col width="20.42578125" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="20.5703125" bestFit="1" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Département </t>
-        </is>
-      </c>
-      <c r="B1" s="36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Type </t>
-        </is>
-      </c>
-      <c r="C1" s="36" t="inlineStr">
-        <is>
-          <t>Intégration avant clôture</t>
-        </is>
-      </c>
-      <c r="D1" s="36" t="inlineStr">
-        <is>
-          <t>Encours de formation</t>
-        </is>
-      </c>
-      <c r="E1" s="37" t="n"/>
-      <c r="F1" s="37" t="n"/>
-      <c r="G1" s="37" t="n"/>
-      <c r="H1" s="37" t="n"/>
-      <c r="I1" s="37" t="n"/>
-      <c r="J1" s="37" t="n"/>
-      <c r="K1" s="37" t="n"/>
-      <c r="L1" s="37" t="n"/>
-      <c r="M1" s="37" t="n"/>
-    </row>
-    <row r="2" ht="15.75" customHeight="1">
-      <c r="A2" s="52" t="n"/>
-      <c r="B2" s="39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Détails </t>
-        </is>
-      </c>
-      <c r="C2" s="39" t="inlineStr">
-        <is>
-          <t>S30</t>
-        </is>
-      </c>
-      <c r="D2" s="39" t="inlineStr">
-        <is>
-          <t>S31</t>
-        </is>
-      </c>
-      <c r="E2" s="40" t="inlineStr">
-        <is>
-          <t>S32</t>
-        </is>
-      </c>
-      <c r="F2" s="40" t="inlineStr">
-        <is>
-          <t>S33</t>
-        </is>
-      </c>
-      <c r="G2" s="40" t="inlineStr">
-        <is>
-          <t>S34</t>
-        </is>
-      </c>
-      <c r="H2" s="40" t="inlineStr">
-        <is>
-          <t>S35</t>
-        </is>
-      </c>
-      <c r="I2" s="40" t="inlineStr">
-        <is>
-          <t>S36</t>
-        </is>
-      </c>
-      <c r="J2" s="40" t="inlineStr">
-        <is>
-          <t>S37</t>
-        </is>
-      </c>
-      <c r="K2" s="40" t="inlineStr">
-        <is>
-          <t>S38</t>
-        </is>
-      </c>
-      <c r="L2" s="40" t="inlineStr">
-        <is>
-          <t>S39</t>
-        </is>
-      </c>
-      <c r="M2" s="40" t="inlineStr">
-        <is>
-          <t>S40</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ferrage  </t>
-        </is>
-      </c>
-      <c r="B3" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Estimation </t>
-        </is>
-      </c>
-      <c r="C3" s="43" t="n">
-        <v>100</v>
-      </c>
-      <c r="D3" s="43" t="n">
-        <v>100</v>
-      </c>
-      <c r="E3" s="44" t="n">
-        <v>100</v>
-      </c>
-      <c r="F3" s="44" t="n">
-        <v>100</v>
-      </c>
-      <c r="G3" s="44" t="n">
-        <v>100</v>
-      </c>
-      <c r="H3" s="44" t="n">
-        <v>100</v>
-      </c>
-      <c r="I3" s="44" t="n">
-        <v>100</v>
-      </c>
-      <c r="J3" s="44" t="n">
-        <v>100</v>
-      </c>
-      <c r="K3" s="44" t="n">
-        <v>100</v>
-      </c>
-      <c r="L3" s="44" t="n">
-        <v>100</v>
-      </c>
-      <c r="M3" s="44" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="53" t="n"/>
-      <c r="B4" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Réel </t>
-        </is>
-      </c>
-      <c r="C4" s="43" t="n">
-        <v>96</v>
-      </c>
-      <c r="D4" s="43" t="n">
-        <v>76</v>
-      </c>
-      <c r="E4" s="44" t="n"/>
-      <c r="F4" s="44" t="n"/>
-      <c r="G4" s="44" t="n"/>
-      <c r="H4" s="44" t="n"/>
-      <c r="I4" s="44" t="n"/>
-      <c r="J4" s="44" t="n"/>
-      <c r="K4" s="44" t="n"/>
-      <c r="L4" s="44" t="n"/>
-      <c r="M4" s="44" t="n"/>
-    </row>
-    <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="52" t="n"/>
-      <c r="B5" s="42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ecart </t>
-        </is>
-      </c>
-      <c r="C5" s="43" t="n">
-        <v>-4</v>
-      </c>
-      <c r="D5" s="43" t="n">
-        <v>-24</v>
-      </c>
-      <c r="E5" s="44" t="n"/>
-      <c r="F5" s="44" t="n"/>
-      <c r="G5" s="44" t="n"/>
-      <c r="H5" s="44" t="n"/>
-      <c r="I5" s="44" t="n"/>
-      <c r="J5" s="44" t="n"/>
-      <c r="K5" s="44" t="n"/>
-      <c r="L5" s="44" t="n"/>
-      <c r="M5" s="44" t="n"/>
-    </row>
-    <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Montage </t>
-        </is>
-      </c>
-      <c r="B6" s="45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Estimation </t>
-        </is>
-      </c>
-      <c r="C6" s="46" t="n">
-        <v>70</v>
-      </c>
-      <c r="D6" s="46" t="n">
-        <v>70</v>
-      </c>
-      <c r="E6" s="47" t="n">
-        <v>70</v>
-      </c>
-      <c r="F6" s="47" t="n">
-        <v>70</v>
-      </c>
-      <c r="G6" s="47" t="n">
-        <v>70</v>
-      </c>
-      <c r="H6" s="47" t="n">
-        <v>70</v>
-      </c>
-      <c r="I6" s="47" t="n">
-        <v>70</v>
-      </c>
-      <c r="J6" s="47" t="n">
-        <v>70</v>
-      </c>
-      <c r="K6" s="47" t="n">
-        <v>70</v>
-      </c>
-      <c r="L6" s="47" t="n">
-        <v>70</v>
-      </c>
-      <c r="M6" s="47" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="53" t="n"/>
-      <c r="B7" s="45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Réel </t>
-        </is>
-      </c>
-      <c r="C7" s="46" t="n">
-        <v>64</v>
-      </c>
-      <c r="D7" s="46" t="n">
-        <v>46</v>
-      </c>
-      <c r="E7" s="47" t="n"/>
-      <c r="F7" s="47" t="n"/>
-      <c r="G7" s="47" t="n"/>
-      <c r="H7" s="47" t="n"/>
-      <c r="I7" s="47" t="n"/>
-      <c r="J7" s="47" t="n"/>
-      <c r="K7" s="47" t="n"/>
-      <c r="L7" s="47" t="n"/>
-      <c r="M7" s="47" t="n"/>
-    </row>
-    <row r="8" ht="15.75" customHeight="1">
-      <c r="A8" s="52" t="n"/>
-      <c r="B8" s="45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ecart </t>
-        </is>
-      </c>
-      <c r="C8" s="46" t="n">
-        <v>-6</v>
-      </c>
-      <c r="D8" s="46" t="n">
-        <v>-24</v>
-      </c>
-      <c r="E8" s="47" t="n"/>
-      <c r="F8" s="47" t="n"/>
-      <c r="G8" s="47" t="n"/>
-      <c r="H8" s="47" t="n"/>
-      <c r="I8" s="47" t="n"/>
-      <c r="J8" s="47" t="n"/>
-      <c r="K8" s="47" t="n"/>
-      <c r="L8" s="47" t="n"/>
-      <c r="M8" s="47" t="n"/>
-    </row>
-    <row r="9" ht="15.75" customHeight="1">
-      <c r="A9" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Peinture </t>
-        </is>
-      </c>
-      <c r="B9" s="48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Estimation </t>
-        </is>
-      </c>
-      <c r="C9" s="49" t="n">
-        <v>20</v>
-      </c>
-      <c r="D9" s="49" t="n">
-        <v>20</v>
-      </c>
-      <c r="E9" s="50" t="n">
-        <v>30</v>
-      </c>
-      <c r="F9" s="50" t="n">
-        <v>20</v>
-      </c>
-      <c r="G9" s="50" t="n">
-        <v>20</v>
-      </c>
-      <c r="H9" s="50" t="n">
-        <v>20</v>
-      </c>
-      <c r="I9" s="50" t="n">
-        <v>20</v>
-      </c>
-      <c r="J9" s="50" t="n">
-        <v>20</v>
-      </c>
-      <c r="K9" s="50" t="n">
-        <v>20</v>
-      </c>
-      <c r="L9" s="50" t="n">
-        <v>20</v>
-      </c>
-      <c r="M9" s="50" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" ht="15.75" customHeight="1">
-      <c r="A10" s="53" t="n"/>
-      <c r="B10" s="48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Réel </t>
-        </is>
-      </c>
-      <c r="C10" s="49" t="n">
+    <row r="4">
+      <c r="B4" s="31" t="inlineStr">
+        <is>
+          <t>Des arrivees IFMIA</t>
+        </is>
+      </c>
+      <c r="F4" s="31" t="inlineStr">
+        <is>
+          <t>Des arrivees Non diplomes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="F5" s="14" t="n"/>
+      <c r="G5" s="10" t="n"/>
+      <c r="H5" s="14" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Effectifs </t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Date Integration IFMIA</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>Date Integration Usine</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>Effectifs</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>Date Integration IFMIA</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Date Integration Usine</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>FER</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="n">
         <v>21</v>
       </c>
-      <c r="D10" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="50" t="n"/>
-      <c r="F10" s="50" t="n"/>
-      <c r="G10" s="50" t="n"/>
-      <c r="H10" s="50" t="n"/>
-      <c r="I10" s="50" t="n"/>
-      <c r="J10" s="50" t="n"/>
-      <c r="K10" s="50" t="n"/>
-      <c r="L10" s="50" t="n"/>
-      <c r="M10" s="50" t="n"/>
-    </row>
-    <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="52" t="n"/>
-      <c r="B11" s="48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ecart </t>
-        </is>
-      </c>
-      <c r="C11" s="49" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="49" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="50" t="n"/>
-      <c r="F11" s="50" t="n"/>
-      <c r="G11" s="50" t="n"/>
-      <c r="H11" s="50" t="n"/>
-      <c r="I11" s="50" t="n"/>
-      <c r="J11" s="50" t="n"/>
-      <c r="K11" s="50" t="n"/>
-      <c r="L11" s="50" t="n"/>
-      <c r="M11" s="50" t="n"/>
-    </row>
-    <row r="12" ht="15.75" customHeight="1">
-      <c r="A12" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total </t>
-        </is>
-      </c>
-      <c r="B12" s="39" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="C12" s="39" t="n">
-        <v>181</v>
-      </c>
-      <c r="D12" s="39" t="n">
-        <v>390</v>
-      </c>
-      <c r="E12" s="40" t="n">
-        <v>590</v>
-      </c>
-      <c r="F12" s="40" t="n">
-        <v>780</v>
-      </c>
-      <c r="G12" s="40" t="n">
-        <v>970</v>
-      </c>
-      <c r="H12" s="40" t="n">
-        <v>1140</v>
-      </c>
-      <c r="I12" s="40" t="n">
-        <v>1310</v>
-      </c>
-      <c r="J12" s="40" t="n">
-        <v>1460</v>
-      </c>
-      <c r="K12" s="40" t="n">
-        <v>1610</v>
-      </c>
-      <c r="L12" s="40" t="n">
-        <v>1710</v>
-      </c>
-      <c r="M12" s="40" t="n">
-        <v>1810</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ecart </t>
-        </is>
-      </c>
-      <c r="B13" s="54" t="n"/>
-      <c r="C13" s="41" t="n">
-        <v>-9</v>
-      </c>
-      <c r="D13" s="41" t="n">
-        <v>-48</v>
-      </c>
-      <c r="E13" s="14" t="n"/>
-      <c r="F13" s="14" t="n"/>
-      <c r="G13" s="14" t="n"/>
-      <c r="H13" s="14" t="n"/>
-      <c r="I13" s="14" t="n"/>
-      <c r="J13" s="14" t="n"/>
-      <c r="K13" s="14" t="n"/>
-      <c r="L13" s="14" t="n"/>
-      <c r="M13" s="14" t="n"/>
+      <c r="C7" s="12" t="n">
+        <v>46239</v>
+      </c>
+      <c r="D7" s="12" t="n">
+        <v>46246</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>MON</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="n">
+        <v>52</v>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>46239</v>
+      </c>
+      <c r="D8" s="12" t="n">
+        <v>46246</v>
+      </c>
+      <c r="F8" s="30" t="n"/>
+      <c r="G8" s="30" t="n"/>
+      <c r="H8" s="30" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="C9" s="12" t="n">
+        <v>46239</v>
+      </c>
+      <c r="D9" s="12" t="n">
+        <v>46253</v>
+      </c>
+      <c r="F9" s="41" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A3:A5"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A6:A8"/>
-    <mergeCell ref="A9:A11"/>
-    <mergeCell ref="A1:A2"/>
+  <mergeCells count="2">
+    <mergeCell ref="F4:I4"/>
+    <mergeCell ref="B4:D4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3484,226 +3158,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="D6:D8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="5" ht="77.25" customHeight="1"/>
-    <row r="6">
-      <c r="D6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nombre d'entrer usine par semaine </t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="D7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total mois </t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="D8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">filtre par S </t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="E8:G8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="8">
-      <c r="E8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">S30 </t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>S31</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>S32</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I25"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
-  <cols>
-    <col width="20.42578125" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="20.5703125" bestFit="1" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1"/>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4">
-      <c r="B4" s="31" t="inlineStr">
-        <is>
-          <t>Des arrivees IFMIA</t>
-        </is>
-      </c>
-      <c r="F4" s="31" t="inlineStr">
-        <is>
-          <t>Des arrivees Non diplomes</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="F5" s="14" t="n"/>
-      <c r="G5" s="10" t="n"/>
-      <c r="H5" s="14" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>UR</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Effectifs </t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>Date Integration IFMIA</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="inlineStr">
-        <is>
-          <t>Date Integration Usine</t>
-        </is>
-      </c>
-      <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>UR</t>
-        </is>
-      </c>
-      <c r="G6" s="14" t="inlineStr">
-        <is>
-          <t>Effectifs</t>
-        </is>
-      </c>
-      <c r="H6" s="14" t="inlineStr">
-        <is>
-          <t>Date Integration IFMIA</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Date Integration Usine</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>FER</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="n">
-        <v>21</v>
-      </c>
-      <c r="C7" s="12" t="n">
-        <v>46239</v>
-      </c>
-      <c r="D7" s="12" t="n">
-        <v>46246</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>MON</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="n">
-        <v>52</v>
-      </c>
-      <c r="C8" s="12" t="n">
-        <v>46239</v>
-      </c>
-      <c r="D8" s="12" t="n">
-        <v>46246</v>
-      </c>
-      <c r="F8" s="30" t="n"/>
-      <c r="G8" s="30" t="n"/>
-      <c r="H8" s="30" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>BC</t>
-        </is>
-      </c>
-      <c r="B9" s="10" t="n">
-        <v>14</v>
-      </c>
-      <c r="C9" s="12" t="n">
-        <v>46239</v>
-      </c>
-      <c r="D9" s="12" t="n">
-        <v>46253</v>
-      </c>
-      <c r="F9" s="41" t="n"/>
-    </row>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="F4:I4"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3771,14 +3226,187 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Appels telephoniques</t>
-        </is>
+          <t>Ferrage - Estimation</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>100</v>
+      </c>
+      <c r="C2" t="n">
+        <v>100</v>
+      </c>
+      <c r="D2" t="n">
+        <v>100</v>
+      </c>
+      <c r="E2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H2" t="n">
+        <v>100</v>
+      </c>
+      <c r="I2" t="n">
+        <v>100</v>
+      </c>
+      <c r="J2" t="n">
+        <v>100</v>
+      </c>
+      <c r="K2" t="n">
+        <v>100</v>
+      </c>
+      <c r="L2" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Ferrage - Reel</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>96</v>
+      </c>
+      <c r="C3" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Montage - Estimation</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>70</v>
+      </c>
+      <c r="C4" t="n">
+        <v>70</v>
+      </c>
+      <c r="D4" t="n">
+        <v>70</v>
+      </c>
+      <c r="E4" t="n">
+        <v>70</v>
+      </c>
+      <c r="F4" t="n">
+        <v>70</v>
+      </c>
+      <c r="G4" t="n">
+        <v>70</v>
+      </c>
+      <c r="H4" t="n">
+        <v>70</v>
+      </c>
+      <c r="I4" t="n">
+        <v>70</v>
+      </c>
+      <c r="J4" t="n">
+        <v>70</v>
+      </c>
+      <c r="K4" t="n">
+        <v>70</v>
+      </c>
+      <c r="L4" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Montage - Reel</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C5" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Peinture - Estimation</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>20</v>
+      </c>
+      <c r="C6" t="n">
+        <v>20</v>
+      </c>
+      <c r="D6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E6" t="n">
+        <v>20</v>
+      </c>
+      <c r="F6" t="n">
+        <v>20</v>
+      </c>
+      <c r="G6" t="n">
+        <v>20</v>
+      </c>
+      <c r="H6" t="n">
+        <v>20</v>
+      </c>
+      <c r="I6" t="n">
+        <v>20</v>
+      </c>
+      <c r="J6" t="n">
+        <v>20</v>
+      </c>
+      <c r="K6" t="n">
+        <v>20</v>
+      </c>
+      <c r="L6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Peinture - Reel</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>21</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Appels telephoniques</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Visite medicale</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Formation IFMIA - Diplomes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Formation IFMIA - Non diplomes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Retire le tableau detail diplomes, ajoute une grille departement x semaine pour les non diplomes
</commit_message>
<xml_diff>
--- a/suivi.xlsx
+++ b/suivi.xlsx
@@ -3025,7 +3025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A4:I9"/>
+  <dimension ref="A4:Q9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="20.42578125" bestFit="1" customWidth="1" min="3" max="3"/>
@@ -3077,17 +3077,57 @@
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>Effectifs</t>
+          <t>S30</t>
         </is>
       </c>
       <c r="H6" s="14" t="inlineStr">
         <is>
-          <t>Date Integration IFMIA</t>
+          <t>S31</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Date Integration Usine</t>
+          <t>S32</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>S33</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>S34</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>S35</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>S36</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>S37</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>S38</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>S39</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>S40</t>
         </is>
       </c>
     </row>
@@ -3105,6 +3145,14 @@
       </c>
       <c r="D7" s="12" t="n">
         <v>46246</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>FER</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>42</v>
       </c>
     </row>
     <row r="8">
@@ -3145,8 +3193,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="F4:I4"/>
     <mergeCell ref="B4:D4"/>
+    <mergeCell ref="F4:Q4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3158,7 +3206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3396,20 +3444,6 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Formation IFMIA - Diplomes</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Formation IFMIA - Non diplomes</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Ajoute le panneau Problematiques identifiees (source Excel)
</commit_message>
<xml_diff>
--- a/suivi.xlsx
+++ b/suivi.xlsx
@@ -9,6 +9,7 @@
     <sheet name="integration Usine" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="En formation IFMIA" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Indicateurs Hebdomadaires" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Problematiques" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'integration Usine'!$B$1:$E$105</definedName>
@@ -3447,4 +3448,62 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Champ</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Valeur</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>La plupart des candidats contactes par telephone presentent l'une des difficultes suivantes : contrat ANAPEC deja consomme, candidature deposee sans reel interet pour le profil operateur, ou quota ANAPEC deja utilise dans sa totalite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Perte visite medicale - formation (%)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Perte durant parcours formation (%)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Ameliore l'UX du panneau Problematiques: liste de raisons scannable + icones
</commit_message>
<xml_diff>
--- a/suivi.xlsx
+++ b/suivi.xlsx
@@ -3456,7 +3456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3474,32 +3474,68 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Intro</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>La plupart des candidats contactes par telephone presentent l'une des difficultes suivantes : contrat ANAPEC deja consomme, candidature deposee sans reel interet pour le profil operateur, ou quota ANAPEC deja utilise dans sa totalite.</t>
+          <t>Constats issus des appels de sourcing candidats</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Perte visite medicale - formation (%)</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>50</v>
+          <t>Raison 1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Contrat ANAPEC deja consomme</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>Raison 2</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Candidature deposee sans reel interet pour le profil operateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Raison 3</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Quota ANAPEC deja utilise dans sa totalite</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Perte visite medicale - formation (%)</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>Perte durant parcours formation (%)</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B7" t="n">
         <v>30</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Calcule le Reel Formation depuis integration Usine, ajoute le tableau Formation par atelier
</commit_message>
<xml_diff>
--- a/suivi.xlsx
+++ b/suivi.xlsx
@@ -3207,7 +3207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3315,131 +3315,92 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ferrage - Reel</t>
+          <t>Montage - Estimation</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>96</v>
+        <v>70</v>
       </c>
       <c r="C3" t="n">
-        <v>76</v>
+        <v>70</v>
+      </c>
+      <c r="D3" t="n">
+        <v>70</v>
+      </c>
+      <c r="E3" t="n">
+        <v>70</v>
+      </c>
+      <c r="F3" t="n">
+        <v>70</v>
+      </c>
+      <c r="G3" t="n">
+        <v>70</v>
+      </c>
+      <c r="H3" t="n">
+        <v>70</v>
+      </c>
+      <c r="I3" t="n">
+        <v>70</v>
+      </c>
+      <c r="J3" t="n">
+        <v>70</v>
+      </c>
+      <c r="K3" t="n">
+        <v>70</v>
+      </c>
+      <c r="L3" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Montage - Estimation</t>
+          <t>Peinture - Estimation</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="C4" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="D4" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="E4" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="F4" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="G4" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="H4" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="I4" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="J4" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="K4" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="L4" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Montage - Reel</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>64</v>
-      </c>
-      <c r="C5" t="n">
-        <v>46</v>
+          <t>Appels telephoniques</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
-        <is>
-          <t>Peinture - Estimation</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>20</v>
-      </c>
-      <c r="C6" t="n">
-        <v>20</v>
-      </c>
-      <c r="D6" t="n">
-        <v>30</v>
-      </c>
-      <c r="E6" t="n">
-        <v>20</v>
-      </c>
-      <c r="F6" t="n">
-        <v>20</v>
-      </c>
-      <c r="G6" t="n">
-        <v>20</v>
-      </c>
-      <c r="H6" t="n">
-        <v>20</v>
-      </c>
-      <c r="I6" t="n">
-        <v>20</v>
-      </c>
-      <c r="J6" t="n">
-        <v>20</v>
-      </c>
-      <c r="K6" t="n">
-        <v>20</v>
-      </c>
-      <c r="L6" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Peinture - Reel</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>21</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Appels telephoniques</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
         <is>
           <t>Visite medicale</t>
         </is>

</xml_diff>

<commit_message>
Ajoute la note NB sous le tableau, valeurs Appels/Visite S32, nettoyage code mort
</commit_message>
<xml_diff>
--- a/suivi.xlsx
+++ b/suivi.xlsx
@@ -3398,12 +3398,18 @@
           <t>Appels telephoniques</t>
         </is>
       </c>
+      <c r="D5" t="n">
+        <v>950</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
           <t>Visite medicale</t>
         </is>
+      </c>
+      <c r="D6" t="n">
+        <v>305</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: ajoute les indicateurs S33 (appels, visite medicale, non diplomes)
Appels telephoniques=100, Visite medicale=50, En formation non diplomes
(total)=35 pour S33, sans toucher aux valeurs historiques de S32.
</commit_message>
<xml_diff>
--- a/suivi.xlsx
+++ b/suivi.xlsx
@@ -3026,13 +3026,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A4:Q9"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="20.42578125" bestFit="1" customWidth="1" min="3" max="3"/>
     <col width="20.5703125" bestFit="1" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
     <row r="4">
       <c r="B4" s="31" t="inlineStr">
         <is>
@@ -3171,9 +3174,16 @@
       <c r="D8" s="12" t="n">
         <v>46246</v>
       </c>
-      <c r="F8" s="30" t="n"/>
+      <c r="F8" s="30" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
       <c r="G8" s="30" t="n"/>
       <c r="H8" s="30" t="n"/>
+      <c r="J8" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -3401,6 +3411,9 @@
       <c r="D5" t="n">
         <v>950</v>
       </c>
+      <c r="E5" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3410,6 +3423,9 @@
       </c>
       <c r="D6" t="n">
         <v>305</v>
+      </c>
+      <c r="E6" t="n">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: arrivees prevues editables + carte Depart IFMIA
- La rubrique "Arrivee prevue" lit desormais la feuille "Arrivees
  Prevues" (Date/Categorie/Valeur), une liste editable a la main plutot
  que deduite du tableau des diplomes. Chaque entree a un crayon pour
  modifier sa valeur et telecharger le fichier mis a jour.
- Ajoute les 3 arrivees annoncees : demain (Diplomes IFMIA, 200),
  mercredi (Non diplomes, 66), jeudi (Diplomes, 67).
- Corrige le filtre de date de la rubrique : elle se basait sur le
  dimanche de la semaine selectionnee (refPoint) et masquait les
  entrees pourtant a venir dans la meme semaine ; utilise maintenant
  le lundi de la semaine (ou aujourd'hui si aucune semaine choisie).
- Nouvelle carte KPI "Depart IFMIA" (hebdomadaire, comme Appels/Visite).
- Met a jour Ferrage (19) et Montage (48) dans le tableau des diplomes.
</commit_message>
<xml_diff>
--- a/suivi.xlsx
+++ b/suivi.xlsx
@@ -10,6 +10,7 @@
     <sheet name="En formation IFMIA" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Indicateurs Hebdomadaires" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Problematiques" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Arrivees Prevues" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'integration Usine'!$B$1:$E$105</definedName>
@@ -20,7 +21,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
+  </numFmts>
   <fonts count="8">
     <font>
       <name val="Aptos Narrow"/>
@@ -352,7 +355,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -505,6 +508,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3142,7 +3147,7 @@
         </is>
       </c>
       <c r="B7" s="10" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C7" s="12" t="n">
         <v>46239</v>
@@ -3166,7 +3171,7 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C8" s="12" t="n">
         <v>46239</v>
@@ -3217,7 +3222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3426,6 +3431,16 @@
       </c>
       <c r="E6" t="n">
         <v>50</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Depart IFMIA</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -3525,4 +3540,74 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Categorie</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Valeur</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="57" t="n">
+        <v>46245</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Diplomes</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="57" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Non diplomes</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="57" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Diplomes</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Total IFMIA devient une valeur manuelle (ligne TOTAL), plus la somme
"En formation total a IFMIA" lit desormais une ligne "TOTAL" dediee
dans la grille UR x semaine, au lieu de sommer Ferrage + Montage + BC.
S33 = 87 (valeur manuelle, distincte des 81 obtenus en additionnant
les ateliers). Ajoute l'edition (crayon) pour cette carte, meme
mecanisme que Ferrage/Montage.
</commit_message>
<xml_diff>
--- a/suivi.xlsx
+++ b/suivi.xlsx
@@ -3031,13 +3031,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A4:Y11"/>
+  <dimension ref="A1:Y10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="20.42578125" bestFit="1" customWidth="1" min="3" max="3"/>
     <col width="20.5703125" bestFit="1" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
@@ -3236,8 +3239,16 @@
       </c>
       <c r="F9" s="41" t="n"/>
     </row>
-    <row r="10"/>
-    <row r="11"/>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>87</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="N4:Y4"/>

</xml_diff>

<commit_message>
update the excel file
</commit_message>
<xml_diff>
--- a/suivi.xlsx
+++ b/suivi.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TA38804\Downloads\dashboard-static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FC92E32-9B80-42CC-9F1C-67F8659ED5B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AF642C5-CCD8-4289-B7CF-B5BBA9B3CE22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2685" yWindow="2685" windowWidth="16890" windowHeight="11295" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2685" yWindow="2685" windowWidth="16890" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="integration Usine" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="67">
   <si>
     <t>Des arrivees Non diplomes</t>
   </si>
@@ -131,9 +131,6 @@
   </si>
   <si>
     <t>EMB APPRENTIS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Montage </t>
   </si>
   <si>
     <t xml:space="preserve">O2X apprentis </t>
@@ -2637,7 +2634,7 @@
     </row>
     <row r="108" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B108" s="15" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="C108" s="15">
         <v>46</v>
@@ -2688,7 +2685,7 @@
     </row>
     <row r="111" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B111" s="15" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C111" s="15">
         <v>6</v>
@@ -2705,7 +2702,7 @@
     </row>
     <row r="112" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B112" s="15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C112" s="15">
         <v>4</v>
@@ -2722,7 +2719,7 @@
     </row>
     <row r="113" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B113" s="15" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C113" s="15">
         <v>4</v>
@@ -2765,7 +2762,7 @@
   <sheetData>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B4" s="35"/>
       <c r="C4" s="35"/>
@@ -2858,7 +2855,7 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -2979,7 +2976,7 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B1" t="s">
         <v>2</v>
@@ -3017,7 +3014,7 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2">
         <v>100</v>
@@ -3055,7 +3052,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B3">
         <v>70</v>
@@ -3093,7 +3090,7 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4">
         <v>20</v>
@@ -3131,7 +3128,7 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D5">
         <v>950</v>
@@ -3142,7 +3139,7 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D6">
         <v>305</v>
@@ -3153,7 +3150,7 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E7">
         <v>30</v>
@@ -3171,47 +3168,47 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" t="s">
         <v>47</v>
-      </c>
-      <c r="B1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" t="s">
         <v>49</v>
-      </c>
-      <c r="B2" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" t="s">
         <v>51</v>
-      </c>
-      <c r="B3" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" t="s">
         <v>53</v>
-      </c>
-      <c r="B4" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" t="s">
         <v>55</v>
-      </c>
-      <c r="B5" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B6">
         <v>50</v>
@@ -3219,7 +3216,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B7">
         <v>30</v>
@@ -3240,13 +3237,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B1" t="s">
         <v>59</v>
       </c>
-      <c r="B1" t="s">
-        <v>60</v>
-      </c>
       <c r="C1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -3254,7 +3251,7 @@
         <v>46245</v>
       </c>
       <c r="B2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C2">
         <v>141</v>
@@ -3265,7 +3262,7 @@
         <v>46246</v>
       </c>
       <c r="B3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C3">
         <v>66</v>
@@ -3276,7 +3273,7 @@
         <v>46247</v>
       </c>
       <c r="B4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C4">
         <v>67</v>
@@ -3297,10 +3294,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B1" t="s">
         <v>63</v>
-      </c>
-      <c r="B1" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -3313,7 +3310,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B3">
         <v>46</v>
@@ -3337,7 +3334,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B6">
         <v>6</v>
@@ -3345,7 +3342,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B7">
         <v>8</v>

</xml_diff>

<commit_message>
same modifications(vedio, text of the card and data)
</commit_message>
<xml_diff>
--- a/suivi.xlsx
+++ b/suivi.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\user\TA38804\Documents\ALL PFE Projects\dashboard-static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C82639B-07CF-4EA3-9BD5-481EDB707658}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77ADC14D-C046-4FBD-926B-1EEB7D123E4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="integration Usine" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="74">
   <si>
     <t>Des arrivees Non diplomes</t>
   </si>
@@ -246,9 +246,6 @@
   </si>
   <si>
     <t xml:space="preserve">Moteur apprentis </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MONTAGE </t>
   </si>
   <si>
     <t>Apprentis montage</t>
@@ -569,8 +566,8 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -905,6 +902,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="B1:F123"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -931,7 +929,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
         <v>19</v>
       </c>
@@ -947,8 +945,8 @@
       <c r="F2" s="16"/>
     </row>
     <row r="3" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="3" t="s">
-        <v>13</v>
+      <c r="B3" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C3" s="4">
         <v>52</v>
@@ -961,9 +959,9 @@
       </c>
       <c r="F3" s="16"/>
     </row>
-    <row r="4" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="3" t="s">
-        <v>20</v>
+    <row r="4" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="15" t="s">
+        <v>73</v>
       </c>
       <c r="C4" s="4">
         <v>46</v>
@@ -976,7 +974,7 @@
       </c>
       <c r="F4" s="16"/>
     </row>
-    <row r="5" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="s">
         <v>21</v>
       </c>
@@ -992,8 +990,8 @@
       <c r="F5" s="16"/>
     </row>
     <row r="6" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="3" t="s">
-        <v>13</v>
+      <c r="B6" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C6" s="4">
         <v>37</v>
@@ -1006,9 +1004,9 @@
       </c>
       <c r="F6" s="16"/>
     </row>
-    <row r="7" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="3" t="s">
-        <v>20</v>
+    <row r="7" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="15" t="s">
+        <v>73</v>
       </c>
       <c r="C7" s="4">
         <v>23</v>
@@ -1021,7 +1019,7 @@
       </c>
       <c r="F7" s="16"/>
     </row>
-    <row r="8" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
         <v>22</v>
       </c>
@@ -1036,7 +1034,7 @@
       </c>
       <c r="F8" s="16"/>
     </row>
-    <row r="9" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
         <v>19</v>
       </c>
@@ -1051,7 +1049,7 @@
       </c>
       <c r="F9" s="16"/>
     </row>
-    <row r="10" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
         <v>22</v>
       </c>
@@ -1066,7 +1064,7 @@
       </c>
       <c r="F10" s="16"/>
     </row>
-    <row r="11" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="3" t="s">
         <v>21</v>
       </c>
@@ -1082,8 +1080,8 @@
       <c r="F11" s="16"/>
     </row>
     <row r="12" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="3" t="s">
-        <v>13</v>
+      <c r="B12" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C12" s="4">
         <v>21</v>
@@ -1096,7 +1094,7 @@
       </c>
       <c r="F12" s="16"/>
     </row>
-    <row r="13" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
         <v>23</v>
       </c>
@@ -1111,9 +1109,9 @@
       </c>
       <c r="F13" s="16"/>
     </row>
-    <row r="14" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="3" t="s">
-        <v>20</v>
+    <row r="14" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="15" t="s">
+        <v>73</v>
       </c>
       <c r="C14" s="4">
         <v>33</v>
@@ -1126,7 +1124,7 @@
       </c>
       <c r="F14" s="16"/>
     </row>
-    <row r="15" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
         <v>19</v>
       </c>
@@ -1142,8 +1140,8 @@
       <c r="F15" s="16"/>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B16" s="4" t="s">
-        <v>13</v>
+      <c r="B16" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C16" s="4">
         <v>27</v>
@@ -1155,9 +1153,9 @@
         <v>46177</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B17" s="4" t="s">
-        <v>20</v>
+    <row r="17" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="15" t="s">
+        <v>73</v>
       </c>
       <c r="C17" s="4">
         <v>26</v>
@@ -1169,7 +1167,7 @@
         <v>46177</v>
       </c>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
         <v>23</v>
       </c>
@@ -1183,7 +1181,7 @@
         <v>46177</v>
       </c>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B19" s="4" t="s">
         <v>19</v>
       </c>
@@ -1198,8 +1196,8 @@
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B20" s="4" t="s">
-        <v>13</v>
+      <c r="B20" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C20" s="4">
         <v>44</v>
@@ -1211,7 +1209,7 @@
         <v>46177</v>
       </c>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B21" s="4" t="s">
         <v>21</v>
       </c>
@@ -1226,8 +1224,8 @@
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B22" s="5" t="s">
-        <v>13</v>
+      <c r="B22" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C22" s="4">
         <v>22</v>
@@ -1239,9 +1237,9 @@
         <v>46183</v>
       </c>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B23" s="5" t="s">
-        <v>20</v>
+    <row r="23" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="15" t="s">
+        <v>73</v>
       </c>
       <c r="C23" s="4">
         <v>22</v>
@@ -1253,7 +1251,7 @@
         <v>46183</v>
       </c>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B24" s="5" t="s">
         <v>23</v>
       </c>
@@ -1267,7 +1265,7 @@
         <v>46183</v>
       </c>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B25" s="5" t="s">
         <v>19</v>
       </c>
@@ -1281,7 +1279,7 @@
         <v>46183</v>
       </c>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B26" s="5" t="s">
         <v>24</v>
       </c>
@@ -1296,8 +1294,8 @@
       </c>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B27" s="5" t="s">
-        <v>13</v>
+      <c r="B27" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C27" s="4">
         <v>28</v>
@@ -1309,9 +1307,9 @@
         <v>46184</v>
       </c>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B28" s="6" t="s">
-        <v>20</v>
+    <row r="28" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="15" t="s">
+        <v>73</v>
       </c>
       <c r="C28" s="7">
         <v>20</v>
@@ -1327,8 +1325,8 @@
       </c>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B29" s="6" t="s">
-        <v>13</v>
+      <c r="B29" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C29" s="7">
         <v>22</v>
@@ -1343,7 +1341,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B30" s="6" t="s">
         <v>19</v>
       </c>
@@ -1360,7 +1358,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B31" s="6" t="s">
         <v>21</v>
       </c>
@@ -1377,7 +1375,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B32" s="6" t="s">
         <v>23</v>
       </c>
@@ -1395,8 +1393,8 @@
       </c>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B33" s="7" t="s">
-        <v>13</v>
+      <c r="B33" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C33" s="7">
         <v>52</v>
@@ -1411,7 +1409,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B34" s="7" t="s">
         <v>23</v>
       </c>
@@ -1428,7 +1426,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B35" s="7" t="s">
         <v>24</v>
       </c>
@@ -1445,7 +1443,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B36" s="7" t="s">
         <v>22</v>
       </c>
@@ -1462,7 +1460,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B37" s="7" t="s">
         <v>19</v>
       </c>
@@ -1479,7 +1477,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B38" s="7" t="s">
         <v>23</v>
       </c>
@@ -1497,8 +1495,8 @@
       </c>
     </row>
     <row r="39" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B39" s="7" t="s">
-        <v>13</v>
+      <c r="B39" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C39" s="7">
         <v>14</v>
@@ -1513,9 +1511,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B40" s="7" t="s">
-        <v>20</v>
+    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="15" t="s">
+        <v>73</v>
       </c>
       <c r="C40" s="7">
         <v>25</v>
@@ -1530,7 +1528,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B41" s="7" t="s">
         <v>19</v>
       </c>
@@ -1547,9 +1545,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B42" s="7" t="s">
-        <v>20</v>
+    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="15" t="s">
+        <v>73</v>
       </c>
       <c r="C42" s="7">
         <v>30</v>
@@ -1564,7 +1562,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B43" s="7" t="s">
         <v>22</v>
       </c>
@@ -1581,7 +1579,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="44" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B44" s="7" t="s">
         <v>21</v>
       </c>
@@ -1598,7 +1596,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="45" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B45" s="7" t="s">
         <v>21</v>
       </c>
@@ -1615,7 +1613,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="46" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B46" s="7" t="s">
         <v>26</v>
       </c>
@@ -1632,7 +1630,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="47" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B47" s="7" t="s">
         <v>27</v>
       </c>
@@ -1650,8 +1648,8 @@
       </c>
     </row>
     <row r="48" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B48" s="7" t="s">
-        <v>13</v>
+      <c r="B48" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C48" s="7">
         <v>23</v>
@@ -1667,8 +1665,8 @@
       </c>
     </row>
     <row r="49" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B49" s="7" t="s">
-        <v>13</v>
+      <c r="B49" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C49" s="7">
         <v>17</v>
@@ -1684,8 +1682,8 @@
       </c>
     </row>
     <row r="50" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B50" s="7" t="s">
-        <v>13</v>
+      <c r="B50" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C50" s="7">
         <v>15</v>
@@ -1701,8 +1699,8 @@
       </c>
     </row>
     <row r="51" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B51" s="7" t="s">
-        <v>13</v>
+      <c r="B51" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C51" s="7">
         <v>1</v>
@@ -1718,8 +1716,8 @@
       </c>
     </row>
     <row r="52" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B52" s="7" t="s">
-        <v>13</v>
+      <c r="B52" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C52" s="7">
         <v>27</v>
@@ -1735,8 +1733,8 @@
       </c>
     </row>
     <row r="53" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B53" s="7" t="s">
-        <v>13</v>
+      <c r="B53" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C53" s="7">
         <v>27</v>
@@ -1752,8 +1750,8 @@
       </c>
     </row>
     <row r="54" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B54" s="7" t="s">
-        <v>13</v>
+      <c r="B54" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C54" s="7">
         <v>27</v>
@@ -1768,9 +1766,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B55" s="9" t="s">
-        <v>20</v>
+    <row r="55" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B55" s="15" t="s">
+        <v>73</v>
       </c>
       <c r="C55" s="7">
         <v>27</v>
@@ -1785,9 +1783,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B56" s="9" t="s">
-        <v>20</v>
+    <row r="56" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B56" s="15" t="s">
+        <v>73</v>
       </c>
       <c r="C56" s="7">
         <v>22</v>
@@ -1802,7 +1800,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="57" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B57" s="9" t="s">
         <v>26</v>
       </c>
@@ -1819,7 +1817,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="58" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B58" s="9" t="s">
         <v>23</v>
       </c>
@@ -1836,7 +1834,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="59" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B59" s="9" t="s">
         <v>23</v>
       </c>
@@ -1853,7 +1851,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="60" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B60" s="9" t="s">
         <v>22</v>
       </c>
@@ -1870,7 +1868,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="61" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B61" s="9" t="s">
         <v>19</v>
       </c>
@@ -1887,7 +1885,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="62" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B62" s="9" t="s">
         <v>19</v>
       </c>
@@ -1904,7 +1902,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="63" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B63" s="9" t="s">
         <v>21</v>
       </c>
@@ -1921,7 +1919,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="64" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B64" s="9" t="s">
         <v>23</v>
       </c>
@@ -1939,8 +1937,8 @@
       </c>
     </row>
     <row r="65" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B65" s="9" t="s">
-        <v>13</v>
+      <c r="B65" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C65" s="9">
         <v>25</v>
@@ -1956,8 +1954,8 @@
       </c>
     </row>
     <row r="66" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B66" s="9" t="s">
-        <v>13</v>
+      <c r="B66" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C66" s="9">
         <v>28</v>
@@ -1972,7 +1970,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="67" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B67" s="9" t="s">
         <v>21</v>
       </c>
@@ -1990,8 +1988,8 @@
       </c>
     </row>
     <row r="68" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B68" s="9" t="s">
-        <v>13</v>
+      <c r="B68" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C68" s="9">
         <v>26</v>
@@ -2006,7 +2004,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="69" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B69" s="9" t="s">
         <v>19</v>
       </c>
@@ -2023,7 +2021,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="70" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B70" s="9" t="s">
         <v>23</v>
       </c>
@@ -2040,7 +2038,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="71" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B71" s="9" t="s">
         <v>26</v>
       </c>
@@ -2057,7 +2055,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="72" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B72" s="9" t="s">
         <v>23</v>
       </c>
@@ -2074,9 +2072,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="73" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B73" s="9" t="s">
-        <v>20</v>
+    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B73" s="15" t="s">
+        <v>73</v>
       </c>
       <c r="C73" s="9">
         <v>62</v>
@@ -2091,7 +2089,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="74" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B74" s="9" t="s">
         <v>21</v>
       </c>
@@ -2109,8 +2107,8 @@
       </c>
     </row>
     <row r="75" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B75" s="9" t="s">
-        <v>13</v>
+      <c r="B75" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C75" s="9">
         <v>63</v>
@@ -2126,8 +2124,8 @@
       </c>
     </row>
     <row r="76" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B76" s="9" t="s">
-        <v>13</v>
+      <c r="B76" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C76" s="9">
         <v>26</v>
@@ -2143,8 +2141,8 @@
       </c>
     </row>
     <row r="77" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B77" s="9" t="s">
-        <v>13</v>
+      <c r="B77" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C77" s="9">
         <v>19</v>
@@ -2159,7 +2157,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="78" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B78" s="9" t="s">
         <v>23</v>
       </c>
@@ -2177,8 +2175,8 @@
       </c>
     </row>
     <row r="79" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B79" s="9" t="s">
-        <v>13</v>
+      <c r="B79" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C79" s="9">
         <v>22</v>
@@ -2194,8 +2192,8 @@
       </c>
     </row>
     <row r="80" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B80" s="9" t="s">
-        <v>13</v>
+      <c r="B80" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C80" s="9">
         <v>13</v>
@@ -2210,7 +2208,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="81" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B81" s="9" t="s">
         <v>27</v>
       </c>
@@ -2227,9 +2225,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B82" s="9" t="s">
-        <v>20</v>
+    <row r="82" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B82" s="15" t="s">
+        <v>73</v>
       </c>
       <c r="C82" s="9">
         <v>34</v>
@@ -2244,7 +2242,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="83" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B83" s="9" t="s">
         <v>23</v>
       </c>
@@ -2262,8 +2260,8 @@
       </c>
     </row>
     <row r="84" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B84" s="12" t="s">
-        <v>13</v>
+      <c r="B84" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C84" s="11">
         <v>14</v>
@@ -2278,7 +2276,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="85" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B85" s="12" t="s">
         <v>22</v>
       </c>
@@ -2295,9 +2293,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B86" s="12" t="s">
-        <v>20</v>
+    <row r="86" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B86" s="15" t="s">
+        <v>73</v>
       </c>
       <c r="C86" s="11">
         <v>17</v>
@@ -2313,8 +2311,8 @@
       </c>
     </row>
     <row r="87" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B87" s="12" t="s">
-        <v>13</v>
+      <c r="B87" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C87" s="12">
         <v>20</v>
@@ -2330,8 +2328,8 @@
       </c>
     </row>
     <row r="88" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B88" s="12" t="s">
-        <v>13</v>
+      <c r="B88" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C88" s="12">
         <v>20</v>
@@ -2346,9 +2344,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B89" s="12" t="s">
-        <v>20</v>
+    <row r="89" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B89" s="15" t="s">
+        <v>73</v>
       </c>
       <c r="C89" s="12">
         <v>18</v>
@@ -2363,7 +2361,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="90" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B90" s="14" t="s">
         <v>30</v>
       </c>
@@ -2380,7 +2378,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="91" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B91" s="12" t="s">
         <v>21</v>
       </c>
@@ -2398,8 +2396,8 @@
       </c>
     </row>
     <row r="92" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B92" s="12" t="s">
-        <v>13</v>
+      <c r="B92" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C92" s="12">
         <v>24</v>
@@ -2414,7 +2412,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="93" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B93" s="12" t="s">
         <v>21</v>
       </c>
@@ -2431,9 +2429,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="94" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B94" s="12" t="s">
-        <v>20</v>
+    <row r="94" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B94" s="15" t="s">
+        <v>73</v>
       </c>
       <c r="C94" s="12">
         <v>17</v>
@@ -2449,8 +2447,8 @@
       </c>
     </row>
     <row r="95" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B95" s="12" t="s">
-        <v>13</v>
+      <c r="B95" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C95" s="12">
         <v>31</v>
@@ -2465,7 +2463,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="96" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B96" s="12" t="s">
         <v>31</v>
       </c>
@@ -2482,7 +2480,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="97" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B97" s="12" t="s">
         <v>32</v>
       </c>
@@ -2499,7 +2497,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="98" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B98" s="12" t="s">
         <v>24</v>
       </c>
@@ -2516,7 +2514,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="99" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B99" s="12" t="s">
         <v>32</v>
       </c>
@@ -2534,8 +2532,8 @@
       </c>
     </row>
     <row r="100" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B100" s="12" t="s">
-        <v>13</v>
+      <c r="B100" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C100" s="12">
         <v>43</v>
@@ -2550,9 +2548,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="101" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B101" s="12" t="s">
-        <v>20</v>
+    <row r="101" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B101" s="15" t="s">
+        <v>73</v>
       </c>
       <c r="C101" s="12">
         <v>12</v>
@@ -2567,7 +2565,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="102" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B102" s="12" t="s">
         <v>23</v>
       </c>
@@ -2584,7 +2582,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="103" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B103" s="12" t="s">
         <v>32</v>
       </c>
@@ -2601,7 +2599,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="104" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B104" s="12" t="s">
         <v>33</v>
       </c>
@@ -2619,8 +2617,8 @@
       </c>
     </row>
     <row r="105" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B105" s="12" t="s">
-        <v>13</v>
+      <c r="B105" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C105" s="12">
         <v>28</v>
@@ -2636,8 +2634,8 @@
       </c>
     </row>
     <row r="106" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B106" s="15" t="s">
-        <v>13</v>
+      <c r="B106" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C106" s="15">
         <v>19</v>
@@ -2653,8 +2651,8 @@
       </c>
     </row>
     <row r="107" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B107" s="15" t="s">
-        <v>13</v>
+      <c r="B107" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C107" s="15">
         <v>37</v>
@@ -2669,9 +2667,9 @@
         <v>28</v>
       </c>
     </row>
-    <row r="108" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B108" s="15" t="s">
-        <v>20</v>
+        <v>73</v>
       </c>
       <c r="C108" s="15">
         <v>46</v>
@@ -2686,7 +2684,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="109" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B109" s="15" t="s">
         <v>21</v>
       </c>
@@ -2703,7 +2701,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="110" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B110" s="15" t="s">
         <v>32</v>
       </c>
@@ -2720,7 +2718,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="111" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B111" s="15" t="s">
         <v>34</v>
       </c>
@@ -2737,7 +2735,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="112" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B112" s="15" t="s">
         <v>35</v>
       </c>
@@ -2754,7 +2752,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="113" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B113" s="15" t="s">
         <v>67</v>
       </c>
@@ -2772,8 +2770,8 @@
       </c>
     </row>
     <row r="114" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B114" s="15" t="s">
-        <v>13</v>
+      <c r="B114" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C114" s="15">
         <v>47</v>
@@ -2788,9 +2786,9 @@
         <v>28</v>
       </c>
     </row>
-    <row r="115" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B115" s="15" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="C115" s="15">
         <v>100</v>
@@ -2805,9 +2803,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="116" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B116" s="15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C116" s="15">
         <v>2</v>
@@ -2822,9 +2820,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="117" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B117" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C117" s="15">
         <v>2</v>
@@ -2839,9 +2837,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="118" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B118" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C118" s="15">
         <v>1</v>
@@ -2856,9 +2854,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="119" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B119" s="15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C119" s="15">
         <v>10</v>
@@ -2873,9 +2871,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="120" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B120" s="15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C120" s="15">
         <v>13</v>
@@ -2891,8 +2889,8 @@
       </c>
     </row>
     <row r="121" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B121" s="36" t="s">
-        <v>73</v>
+      <c r="B121" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C121" s="15">
         <v>13</v>
@@ -2905,8 +2903,8 @@
       </c>
     </row>
     <row r="122" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B122" s="36" t="s">
-        <v>73</v>
+      <c r="B122" s="35" t="s">
+        <v>72</v>
       </c>
       <c r="C122" s="15">
         <v>60</v>
@@ -2918,9 +2916,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="123" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B123" s="15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C123" s="15">
         <v>36</v>
@@ -2933,7 +2931,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B1:E123" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="B1:E123" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Ferrage"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2948,20 +2952,20 @@
   </cols>
   <sheetData>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="35" t="s">
+      <c r="A4" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="35"/>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="35"/>
-      <c r="F4" s="35"/>
-      <c r="G4" s="35"/>
-      <c r="H4" s="35"/>
-      <c r="I4" s="35"/>
-      <c r="J4" s="35"/>
-      <c r="K4" s="35"/>
-      <c r="L4" s="35"/>
+      <c r="B4" s="36"/>
+      <c r="C4" s="36"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="36"/>
+      <c r="F4" s="36"/>
+      <c r="G4" s="36"/>
+      <c r="H4" s="36"/>
+      <c r="I4" s="36"/>
+      <c r="J4" s="36"/>
+      <c r="K4" s="36"/>
+      <c r="L4" s="36"/>
     </row>
     <row r="5" spans="1:12" s="33" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G5" s="34"/>

</xml_diff>

<commit_message>
update the estimation values
</commit_message>
<xml_diff>
--- a/suivi.xlsx
+++ b/suivi.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\user\TA38804\Documents\ALL PFE Projects\dashboard-static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77ADC14D-C046-4FBD-926B-1EEB7D123E4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22634D2C-74CF-461E-95DE-E4240505870D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="integration Usine" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="73">
   <si>
     <t>Des arrivees Non diplomes</t>
   </si>
@@ -260,10 +260,7 @@
     <t xml:space="preserve">bird cage </t>
   </si>
   <si>
-    <t xml:space="preserve">Ferrage </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Montage </t>
+    <t xml:space="preserve">FER </t>
   </si>
 </sst>
 </file>
@@ -944,7 +941,7 @@
       </c>
       <c r="F2" s="16"/>
     </row>
-    <row r="3" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="35" t="s">
         <v>72</v>
       </c>
@@ -959,9 +956,9 @@
       </c>
       <c r="F3" s="16"/>
     </row>
-    <row r="4" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="15" t="s">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="C4" s="4">
         <v>46</v>
@@ -989,7 +986,7 @@
       </c>
       <c r="F5" s="16"/>
     </row>
-    <row r="6" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="35" t="s">
         <v>72</v>
       </c>
@@ -1004,9 +1001,9 @@
       </c>
       <c r="F6" s="16"/>
     </row>
-    <row r="7" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="15" t="s">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="C7" s="4">
         <v>23</v>
@@ -1079,7 +1076,7 @@
       </c>
       <c r="F11" s="16"/>
     </row>
-    <row r="12" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="35" t="s">
         <v>72</v>
       </c>
@@ -1109,9 +1106,9 @@
       </c>
       <c r="F13" s="16"/>
     </row>
-    <row r="14" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="15" t="s">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="C14" s="4">
         <v>33</v>
@@ -1139,7 +1136,7 @@
       </c>
       <c r="F15" s="16"/>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B16" s="35" t="s">
         <v>72</v>
       </c>
@@ -1153,9 +1150,9 @@
         <v>46177</v>
       </c>
     </row>
-    <row r="17" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="15" t="s">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="C17" s="4">
         <v>26</v>
@@ -1195,7 +1192,7 @@
         <v>46177</v>
       </c>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B20" s="35" t="s">
         <v>72</v>
       </c>
@@ -1223,7 +1220,7 @@
         <v>46178</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B22" s="35" t="s">
         <v>72</v>
       </c>
@@ -1237,9 +1234,9 @@
         <v>46183</v>
       </c>
     </row>
-    <row r="23" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" s="15" t="s">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="C23" s="4">
         <v>22</v>
@@ -1293,7 +1290,7 @@
         <v>46183</v>
       </c>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B27" s="35" t="s">
         <v>72</v>
       </c>
@@ -1307,9 +1304,9 @@
         <v>46184</v>
       </c>
     </row>
-    <row r="28" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28" s="15" t="s">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="C28" s="7">
         <v>20</v>
@@ -1324,7 +1321,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B29" s="35" t="s">
         <v>72</v>
       </c>
@@ -1392,7 +1389,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B33" s="35" t="s">
         <v>72</v>
       </c>
@@ -1494,7 +1491,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B39" s="35" t="s">
         <v>72</v>
       </c>
@@ -1511,9 +1508,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B40" s="15" t="s">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="C40" s="7">
         <v>25</v>
@@ -1545,9 +1542,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B42" s="15" t="s">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="C42" s="7">
         <v>30</v>
@@ -1647,7 +1644,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="48" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B48" s="35" t="s">
         <v>72</v>
       </c>
@@ -1664,7 +1661,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="49" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B49" s="35" t="s">
         <v>72</v>
       </c>
@@ -1681,7 +1678,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="50" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B50" s="35" t="s">
         <v>72</v>
       </c>
@@ -1698,7 +1695,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="51" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B51" s="35" t="s">
         <v>72</v>
       </c>
@@ -1715,7 +1712,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="52" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B52" s="35" t="s">
         <v>72</v>
       </c>
@@ -1732,7 +1729,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="53" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B53" s="35" t="s">
         <v>72</v>
       </c>
@@ -1749,7 +1746,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="54" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B54" s="35" t="s">
         <v>72</v>
       </c>
@@ -1766,9 +1763,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="55" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B55" s="15" t="s">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="C55" s="7">
         <v>27</v>
@@ -1783,9 +1780,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="56" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B56" s="15" t="s">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="C56" s="7">
         <v>22</v>
@@ -1936,7 +1933,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="65" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B65" s="35" t="s">
         <v>72</v>
       </c>
@@ -1953,7 +1950,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="66" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B66" s="35" t="s">
         <v>72</v>
       </c>
@@ -1987,7 +1984,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="68" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B68" s="35" t="s">
         <v>72</v>
       </c>
@@ -2072,9 +2069,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B73" s="15" t="s">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="C73" s="9">
         <v>62</v>
@@ -2106,7 +2103,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="75" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B75" s="35" t="s">
         <v>72</v>
       </c>
@@ -2123,7 +2120,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="76" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B76" s="35" t="s">
         <v>72</v>
       </c>
@@ -2140,7 +2137,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="77" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B77" s="35" t="s">
         <v>72</v>
       </c>
@@ -2174,7 +2171,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="79" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B79" s="35" t="s">
         <v>72</v>
       </c>
@@ -2191,7 +2188,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="80" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B80" s="35" t="s">
         <v>72</v>
       </c>
@@ -2225,9 +2222,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="82" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B82" s="15" t="s">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="C82" s="9">
         <v>34</v>
@@ -2259,7 +2256,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="84" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B84" s="35" t="s">
         <v>72</v>
       </c>
@@ -2293,9 +2290,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="86" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B86" s="15" t="s">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="C86" s="11">
         <v>17</v>
@@ -2310,7 +2307,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="87" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B87" s="35" t="s">
         <v>72</v>
       </c>
@@ -2327,7 +2324,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="88" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B88" s="35" t="s">
         <v>72</v>
       </c>
@@ -2344,9 +2341,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="89" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B89" s="15" t="s">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="C89" s="12">
         <v>18</v>
@@ -2395,7 +2392,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="92" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B92" s="35" t="s">
         <v>72</v>
       </c>
@@ -2429,9 +2426,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="94" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B94" s="15" t="s">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="C94" s="12">
         <v>17</v>
@@ -2446,7 +2443,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="95" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B95" s="35" t="s">
         <v>72</v>
       </c>
@@ -2531,7 +2528,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="100" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B100" s="35" t="s">
         <v>72</v>
       </c>
@@ -2548,9 +2545,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="101" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B101" s="15" t="s">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="C101" s="12">
         <v>12</v>
@@ -2616,7 +2613,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="105" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B105" s="35" t="s">
         <v>72</v>
       </c>
@@ -2633,7 +2630,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="106" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B106" s="35" t="s">
         <v>72</v>
       </c>
@@ -2650,7 +2647,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="107" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B107" s="35" t="s">
         <v>72</v>
       </c>
@@ -2667,9 +2664,9 @@
         <v>28</v>
       </c>
     </row>
-    <row r="108" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B108" s="15" t="s">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="C108" s="15">
         <v>46</v>
@@ -2769,7 +2766,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="114" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B114" s="35" t="s">
         <v>72</v>
       </c>
@@ -2786,9 +2783,9 @@
         <v>28</v>
       </c>
     </row>
-    <row r="115" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B115" s="15" t="s">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="C115" s="15">
         <v>100</v>
@@ -2888,7 +2885,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="121" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B121" s="35" t="s">
         <v>72</v>
       </c>
@@ -2902,7 +2899,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="122" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B122" s="35" t="s">
         <v>72</v>
       </c>
@@ -2916,9 +2913,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="123" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B123" s="15" t="s">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="C123" s="15">
         <v>36</v>
@@ -2934,7 +2931,7 @@
   <autoFilter ref="B1:E123" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="0">
       <filters>
-        <filter val="Ferrage"/>
+        <filter val="Montage"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -3295,10 +3292,10 @@
         <v>20</v>
       </c>
       <c r="D4">
+        <v>20</v>
+      </c>
+      <c r="E4">
         <v>30</v>
-      </c>
-      <c r="E4">
-        <v>20</v>
       </c>
       <c r="F4">
         <v>20</v>

</xml_diff>

<commit_message>
UPDATA THE EXCEL FILE
</commit_message>
<xml_diff>
--- a/suivi.xlsx
+++ b/suivi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\user\TA38804\Documents\ALL PFE Projects\dashboard-static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEF0DECB-47D5-47E6-88AF-16582FB2C67A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0961E2C-DD43-4E9B-98E1-3A2659C183ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
     <sheet name="Repartition Arrivee Usine" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'integration Usine'!$B$1:$E$123</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'integration Usine'!$B$1:$E$136</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="78">
   <si>
     <t>Des arrivees Non diplomes</t>
   </si>
@@ -245,12 +245,6 @@
     <t>Moteur apprentis</t>
   </si>
   <si>
-    <t xml:space="preserve">Moteur apprentis </t>
-  </si>
-  <si>
-    <t>Apprentis montage</t>
-  </si>
-  <si>
     <t>Apprentis UTEE</t>
   </si>
   <si>
@@ -264,6 +258,24 @@
   </si>
   <si>
     <t>Vivier</t>
+  </si>
+  <si>
+    <t>BIRD CAGE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apprentis monteur  </t>
+  </si>
+  <si>
+    <t>PEINTURE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O2X BATTERIE </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MOTEUR </t>
+  </si>
+  <si>
+    <t>APPRENTIS O2X</t>
   </si>
 </sst>
 </file>
@@ -472,7 +484,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -568,7 +580,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -904,7 +915,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="B1:F123"/>
+  <dimension ref="B1:F136"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="15" customWidth="1"/>
@@ -947,7 +958,7 @@
     </row>
     <row r="3" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C3" s="4">
         <v>52</v>
@@ -960,7 +971,7 @@
       </c>
       <c r="F3" s="16"/>
     </row>
-    <row r="4" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="15" t="s">
         <v>20</v>
       </c>
@@ -992,7 +1003,7 @@
     </row>
     <row r="6" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C6" s="4">
         <v>37</v>
@@ -1005,7 +1016,7 @@
       </c>
       <c r="F6" s="16"/>
     </row>
-    <row r="7" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="15" t="s">
         <v>20</v>
       </c>
@@ -1082,7 +1093,7 @@
     </row>
     <row r="12" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C12" s="4">
         <v>21</v>
@@ -1110,7 +1121,7 @@
       </c>
       <c r="F13" s="16"/>
     </row>
-    <row r="14" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="15" t="s">
         <v>20</v>
       </c>
@@ -1142,7 +1153,7 @@
     </row>
     <row r="16" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B16" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C16" s="4">
         <v>27</v>
@@ -1154,7 +1165,7 @@
         <v>46177</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B17" s="15" t="s">
         <v>20</v>
       </c>
@@ -1198,7 +1209,7 @@
     </row>
     <row r="20" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B20" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C20" s="4">
         <v>44</v>
@@ -1226,7 +1237,7 @@
     </row>
     <row r="22" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B22" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C22" s="4">
         <v>22</v>
@@ -1238,7 +1249,7 @@
         <v>46183</v>
       </c>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B23" s="15" t="s">
         <v>20</v>
       </c>
@@ -1296,7 +1307,7 @@
     </row>
     <row r="27" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B27" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C27" s="4">
         <v>28</v>
@@ -1308,7 +1319,7 @@
         <v>46184</v>
       </c>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B28" s="15" t="s">
         <v>20</v>
       </c>
@@ -1327,7 +1338,7 @@
     </row>
     <row r="29" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B29" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C29" s="7">
         <v>22</v>
@@ -1395,7 +1406,7 @@
     </row>
     <row r="33" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B33" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C33" s="7">
         <v>52</v>
@@ -1497,7 +1508,7 @@
     </row>
     <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B39" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C39" s="7">
         <v>14</v>
@@ -1512,7 +1523,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B40" s="15" t="s">
         <v>20</v>
       </c>
@@ -1546,7 +1557,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B42" s="15" t="s">
         <v>20</v>
       </c>
@@ -1650,7 +1661,7 @@
     </row>
     <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B48" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C48" s="7">
         <v>23</v>
@@ -1667,7 +1678,7 @@
     </row>
     <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B49" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C49" s="7">
         <v>17</v>
@@ -1684,7 +1695,7 @@
     </row>
     <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B50" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C50" s="7">
         <v>15</v>
@@ -1701,7 +1712,7 @@
     </row>
     <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B51" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C51" s="7">
         <v>1</v>
@@ -1718,7 +1729,7 @@
     </row>
     <row r="52" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B52" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C52" s="7">
         <v>27</v>
@@ -1735,7 +1746,7 @@
     </row>
     <row r="53" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B53" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C53" s="7">
         <v>27</v>
@@ -1752,7 +1763,7 @@
     </row>
     <row r="54" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B54" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C54" s="7">
         <v>27</v>
@@ -1767,7 +1778,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="55" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B55" s="15" t="s">
         <v>20</v>
       </c>
@@ -1784,7 +1795,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="56" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B56" s="15" t="s">
         <v>20</v>
       </c>
@@ -1939,7 +1950,7 @@
     </row>
     <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B65" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C65" s="9">
         <v>25</v>
@@ -1956,7 +1967,7 @@
     </row>
     <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B66" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C66" s="9">
         <v>28</v>
@@ -1990,7 +2001,7 @@
     </row>
     <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B68" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C68" s="9">
         <v>26</v>
@@ -2073,7 +2084,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="73" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B73" s="15" t="s">
         <v>20</v>
       </c>
@@ -2109,7 +2120,7 @@
     </row>
     <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B75" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C75" s="9">
         <v>63</v>
@@ -2126,7 +2137,7 @@
     </row>
     <row r="76" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B76" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C76" s="9">
         <v>26</v>
@@ -2143,7 +2154,7 @@
     </row>
     <row r="77" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B77" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C77" s="9">
         <v>19</v>
@@ -2177,7 +2188,7 @@
     </row>
     <row r="79" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B79" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C79" s="9">
         <v>22</v>
@@ -2194,7 +2205,7 @@
     </row>
     <row r="80" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B80" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C80" s="9">
         <v>13</v>
@@ -2226,7 +2237,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="82" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B82" s="15" t="s">
         <v>20</v>
       </c>
@@ -2262,7 +2273,7 @@
     </row>
     <row r="84" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B84" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C84" s="11">
         <v>14</v>
@@ -2294,7 +2305,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="86" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B86" s="15" t="s">
         <v>20</v>
       </c>
@@ -2313,7 +2324,7 @@
     </row>
     <row r="87" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B87" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C87" s="12">
         <v>20</v>
@@ -2330,7 +2341,7 @@
     </row>
     <row r="88" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B88" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C88" s="12">
         <v>20</v>
@@ -2345,7 +2356,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="89" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B89" s="15" t="s">
         <v>20</v>
       </c>
@@ -2398,7 +2409,7 @@
     </row>
     <row r="92" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B92" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C92" s="12">
         <v>24</v>
@@ -2430,7 +2441,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="94" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B94" s="15" t="s">
         <v>20</v>
       </c>
@@ -2449,7 +2460,7 @@
     </row>
     <row r="95" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B95" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C95" s="12">
         <v>31</v>
@@ -2534,7 +2545,7 @@
     </row>
     <row r="100" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B100" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C100" s="12">
         <v>43</v>
@@ -2549,7 +2560,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="101" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B101" s="15" t="s">
         <v>20</v>
       </c>
@@ -2619,7 +2630,7 @@
     </row>
     <row r="105" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B105" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C105" s="12">
         <v>28</v>
@@ -2636,7 +2647,7 @@
     </row>
     <row r="106" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B106" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C106" s="15">
         <v>19</v>
@@ -2653,7 +2664,7 @@
     </row>
     <row r="107" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B107" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C107" s="15">
         <v>37</v>
@@ -2668,7 +2679,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="108" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B108" s="15" t="s">
         <v>20</v>
       </c>
@@ -2736,7 +2747,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="112" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B112" s="15" t="s">
         <v>35</v>
       </c>
@@ -2754,8 +2765,8 @@
       </c>
     </row>
     <row r="113" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B113" s="15" t="s">
-        <v>67</v>
+      <c r="B113" s="12" t="s">
+        <v>73</v>
       </c>
       <c r="C113" s="15">
         <v>4</v>
@@ -2772,7 +2783,7 @@
     </row>
     <row r="114" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B114" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C114" s="15">
         <v>47</v>
@@ -2787,7 +2798,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="115" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B115" s="15" t="s">
         <v>20</v>
       </c>
@@ -2804,9 +2815,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="116" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B116" s="15" t="s">
-        <v>68</v>
+        <v>35</v>
       </c>
       <c r="C116" s="15">
         <v>2</v>
@@ -2823,7 +2834,7 @@
     </row>
     <row r="117" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B117" s="15" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C117" s="15">
         <v>2</v>
@@ -2840,7 +2851,7 @@
     </row>
     <row r="118" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B118" s="15" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C118" s="15">
         <v>1</v>
@@ -2857,7 +2868,7 @@
     </row>
     <row r="119" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B119" s="15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C119" s="15">
         <v>10</v>
@@ -2874,7 +2885,7 @@
     </row>
     <row r="120" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B120" s="15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C120" s="15">
         <v>13</v>
@@ -2891,7 +2902,7 @@
     </row>
     <row r="121" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B121" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C121" s="15">
         <v>13</v>
@@ -2905,7 +2916,7 @@
     </row>
     <row r="122" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B122" s="35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C122" s="15">
         <v>60</v>
@@ -2917,7 +2928,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="123" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B123" s="15" t="s">
         <v>20</v>
       </c>
@@ -2931,11 +2942,233 @@
         <v>25</v>
       </c>
     </row>
+    <row r="124" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B124" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="C124" s="12">
+        <v>8</v>
+      </c>
+      <c r="D124" s="24">
+        <v>46256</v>
+      </c>
+      <c r="E124" s="24">
+        <v>46273</v>
+      </c>
+      <c r="F124" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="125" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B125" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="C125" s="12">
+        <v>10</v>
+      </c>
+      <c r="D125" s="24">
+        <v>46258</v>
+      </c>
+      <c r="E125" s="24">
+        <v>46273</v>
+      </c>
+      <c r="F125" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="126" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B126" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C126" s="12">
+        <v>1</v>
+      </c>
+      <c r="D126" s="24">
+        <v>46258</v>
+      </c>
+      <c r="E126" s="24">
+        <v>46273</v>
+      </c>
+      <c r="F126" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="127" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B127" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C127" s="12">
+        <v>1</v>
+      </c>
+      <c r="D127" s="24">
+        <v>46258</v>
+      </c>
+      <c r="E127" s="24">
+        <v>46273</v>
+      </c>
+      <c r="F127" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="128" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B128" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="C128" s="12">
+        <v>58</v>
+      </c>
+      <c r="D128" s="24">
+        <v>46255</v>
+      </c>
+      <c r="E128" s="24">
+        <v>46272</v>
+      </c>
+      <c r="F128" s="12" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="129" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B129" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="C129" s="12">
+        <v>47</v>
+      </c>
+      <c r="D129" s="24">
+        <v>46261</v>
+      </c>
+      <c r="E129" s="24">
+        <v>46276</v>
+      </c>
+      <c r="F129" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="130" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B130" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="C130" s="12">
+        <v>10</v>
+      </c>
+      <c r="D130" s="24">
+        <v>46262</v>
+      </c>
+      <c r="E130" s="24">
+        <v>46276</v>
+      </c>
+      <c r="F130" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="131" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B131" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C131" s="12">
+        <v>42</v>
+      </c>
+      <c r="D131" s="24">
+        <v>46265</v>
+      </c>
+      <c r="E131" s="24">
+        <v>46280</v>
+      </c>
+      <c r="F131" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="132" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B132" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C132" s="12">
+        <v>6</v>
+      </c>
+      <c r="D132" s="24">
+        <v>46265</v>
+      </c>
+      <c r="E132" s="24">
+        <v>46280</v>
+      </c>
+      <c r="F132" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="133" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B133" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="C133" s="12">
+        <v>10</v>
+      </c>
+      <c r="D133" s="24">
+        <v>46265</v>
+      </c>
+      <c r="E133" s="24">
+        <v>46280</v>
+      </c>
+      <c r="F133" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="134" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B134" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="C134" s="12">
+        <v>29</v>
+      </c>
+      <c r="D134" s="24">
+        <v>46265</v>
+      </c>
+      <c r="E134" s="24">
+        <v>46280</v>
+      </c>
+      <c r="F134" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="135" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B135" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="C135" s="12">
+        <v>1</v>
+      </c>
+      <c r="D135" s="24">
+        <v>46265</v>
+      </c>
+      <c r="E135" s="24">
+        <v>46280</v>
+      </c>
+      <c r="F135" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="136" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B136" s="35" t="s">
+        <v>70</v>
+      </c>
+      <c r="C136" s="15">
+        <v>48</v>
+      </c>
+      <c r="D136" s="25">
+        <v>46266</v>
+      </c>
+      <c r="E136" s="25">
+        <v>46281</v>
+      </c>
+      <c r="F136" s="15" t="s">
+        <v>29</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="B1:E123" xr:uid="{00000000-0009-0000-0000-000000000000}">
+  <autoFilter ref="B1:E136" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="0">
       <filters>
-        <filter val="Montage"/>
+        <filter val="APPRENTIS MOTNAGE"/>
+        <filter val="Montage apprentis"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -3039,7 +3272,7 @@
       <c r="E8" s="13">
         <v>96</v>
       </c>
-      <c r="F8" s="37">
+      <c r="F8" s="31">
         <v>54</v>
       </c>
       <c r="G8" s="32"/>
@@ -3302,10 +3535,10 @@
         <v>20</v>
       </c>
       <c r="D4">
+        <v>30</v>
+      </c>
+      <c r="E4">
         <v>20</v>
-      </c>
-      <c r="E4">
-        <v>30</v>
       </c>
       <c r="F4">
         <v>20</v>
@@ -3370,7 +3603,7 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F8">
         <v>330</v>

</xml_diff>

<commit_message>
UPDATA THE EXCEL FILE and the bilan-forum.js
</commit_message>
<xml_diff>
--- a/suivi.xlsx
+++ b/suivi.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\user\TA38804\Documents\ALL PFE Projects\dashboard-static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0961E2C-DD43-4E9B-98E1-3A2659C183ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C269CE5B-3051-42C2-B2EC-514DE0D4D1D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="integration Usine" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="73">
   <si>
     <t>Des arrivees Non diplomes</t>
   </si>
@@ -149,9 +149,6 @@
     <t xml:space="preserve">O2X apprentis </t>
   </si>
   <si>
-    <t xml:space="preserve">Montage apprentis </t>
-  </si>
-  <si>
     <t>Des arrivees IFMIA (par semaine)</t>
   </si>
   <si>
@@ -245,15 +242,6 @@
     <t>Moteur apprentis</t>
   </si>
   <si>
-    <t>Apprentis UTEE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Apprentis emboutissage </t>
-  </si>
-  <si>
-    <t xml:space="preserve">bird cage </t>
-  </si>
-  <si>
     <t xml:space="preserve">FER </t>
   </si>
   <si>
@@ -263,19 +251,16 @@
     <t>BIRD CAGE</t>
   </si>
   <si>
-    <t xml:space="preserve">Apprentis monteur  </t>
-  </si>
-  <si>
-    <t>PEINTURE</t>
-  </si>
-  <si>
     <t xml:space="preserve">O2X BATTERIE </t>
   </si>
   <si>
-    <t xml:space="preserve">MOTEUR </t>
-  </si>
-  <si>
-    <t>APPRENTIS O2X</t>
+    <t xml:space="preserve">Monteur Apprentis </t>
+  </si>
+  <si>
+    <t xml:space="preserve">UTEE APPRENTIS </t>
+  </si>
+  <si>
+    <t>NOn</t>
   </si>
 </sst>
 </file>
@@ -958,7 +943,7 @@
     </row>
     <row r="3" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C3" s="4">
         <v>52</v>
@@ -1003,7 +988,7 @@
     </row>
     <row r="6" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C6" s="4">
         <v>37</v>
@@ -1093,7 +1078,7 @@
     </row>
     <row r="12" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C12" s="4">
         <v>21</v>
@@ -1153,7 +1138,7 @@
     </row>
     <row r="16" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B16" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C16" s="4">
         <v>27</v>
@@ -1209,7 +1194,7 @@
     </row>
     <row r="20" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B20" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C20" s="4">
         <v>44</v>
@@ -1237,7 +1222,7 @@
     </row>
     <row r="22" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B22" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C22" s="4">
         <v>22</v>
@@ -1307,7 +1292,7 @@
     </row>
     <row r="27" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B27" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C27" s="4">
         <v>28</v>
@@ -1338,7 +1323,7 @@
     </row>
     <row r="29" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B29" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C29" s="7">
         <v>22</v>
@@ -1406,7 +1391,7 @@
     </row>
     <row r="33" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B33" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C33" s="7">
         <v>52</v>
@@ -1508,7 +1493,7 @@
     </row>
     <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B39" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C39" s="7">
         <v>14</v>
@@ -1661,7 +1646,7 @@
     </row>
     <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B48" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C48" s="7">
         <v>23</v>
@@ -1678,7 +1663,7 @@
     </row>
     <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B49" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C49" s="7">
         <v>17</v>
@@ -1695,7 +1680,7 @@
     </row>
     <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B50" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C50" s="7">
         <v>15</v>
@@ -1712,7 +1697,7 @@
     </row>
     <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B51" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C51" s="7">
         <v>1</v>
@@ -1729,7 +1714,7 @@
     </row>
     <row r="52" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B52" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C52" s="7">
         <v>27</v>
@@ -1746,7 +1731,7 @@
     </row>
     <row r="53" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B53" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C53" s="7">
         <v>27</v>
@@ -1763,7 +1748,7 @@
     </row>
     <row r="54" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B54" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C54" s="7">
         <v>27</v>
@@ -1950,7 +1935,7 @@
     </row>
     <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B65" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C65" s="9">
         <v>25</v>
@@ -1967,7 +1952,7 @@
     </row>
     <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B66" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C66" s="9">
         <v>28</v>
@@ -2001,7 +1986,7 @@
     </row>
     <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B68" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C68" s="9">
         <v>26</v>
@@ -2120,7 +2105,7 @@
     </row>
     <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B75" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C75" s="9">
         <v>63</v>
@@ -2137,7 +2122,7 @@
     </row>
     <row r="76" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B76" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C76" s="9">
         <v>26</v>
@@ -2154,7 +2139,7 @@
     </row>
     <row r="77" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B77" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C77" s="9">
         <v>19</v>
@@ -2188,7 +2173,7 @@
     </row>
     <row r="79" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B79" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C79" s="9">
         <v>22</v>
@@ -2205,7 +2190,7 @@
     </row>
     <row r="80" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B80" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C80" s="9">
         <v>13</v>
@@ -2273,7 +2258,7 @@
     </row>
     <row r="84" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B84" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C84" s="11">
         <v>14</v>
@@ -2324,7 +2309,7 @@
     </row>
     <row r="87" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B87" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C87" s="12">
         <v>20</v>
@@ -2341,7 +2326,7 @@
     </row>
     <row r="88" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B88" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C88" s="12">
         <v>20</v>
@@ -2409,7 +2394,7 @@
     </row>
     <row r="92" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B92" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C92" s="12">
         <v>24</v>
@@ -2460,7 +2445,7 @@
     </row>
     <row r="95" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B95" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C95" s="12">
         <v>31</v>
@@ -2475,7 +2460,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="96" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B96" s="12" t="s">
         <v>31</v>
       </c>
@@ -2545,7 +2530,7 @@
     </row>
     <row r="100" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B100" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C100" s="12">
         <v>43</v>
@@ -2578,7 +2563,7 @@
       </c>
     </row>
     <row r="102" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B102" s="12" t="s">
+      <c r="B102" s="9" t="s">
         <v>23</v>
       </c>
       <c r="C102" s="12">
@@ -2630,7 +2615,7 @@
     </row>
     <row r="105" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B105" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C105" s="12">
         <v>28</v>
@@ -2647,7 +2632,7 @@
     </row>
     <row r="106" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B106" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C106" s="15">
         <v>19</v>
@@ -2664,7 +2649,7 @@
     </row>
     <row r="107" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B107" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C107" s="15">
         <v>37</v>
@@ -2714,19 +2699,19 @@
       </c>
     </row>
     <row r="110" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B110" s="15" t="s">
+      <c r="B110" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="C110" s="15">
+      <c r="C110" s="12">
         <v>1</v>
       </c>
-      <c r="D110" s="25">
+      <c r="D110" s="24">
         <v>46246</v>
       </c>
-      <c r="E110" s="25">
+      <c r="E110" s="24">
         <v>46265</v>
       </c>
-      <c r="F110" s="15" t="s">
+      <c r="F110" s="12" t="s">
         <v>25</v>
       </c>
     </row>
@@ -2748,8 +2733,8 @@
       </c>
     </row>
     <row r="112" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B112" s="15" t="s">
-        <v>35</v>
+      <c r="B112" s="12" t="s">
+        <v>31</v>
       </c>
       <c r="C112" s="15">
         <v>4</v>
@@ -2765,8 +2750,8 @@
       </c>
     </row>
     <row r="113" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B113" s="12" t="s">
-        <v>73</v>
+      <c r="B113" s="15" t="s">
+        <v>70</v>
       </c>
       <c r="C113" s="15">
         <v>4</v>
@@ -2781,170 +2766,179 @@
         <v>25</v>
       </c>
     </row>
-    <row r="114" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B114" s="35" t="s">
-        <v>70</v>
-      </c>
-      <c r="C114" s="15">
-        <v>47</v>
-      </c>
-      <c r="D114" s="25">
-        <v>46251</v>
-      </c>
-      <c r="E114" s="25">
-        <v>46268</v>
-      </c>
-      <c r="F114" s="15" t="s">
-        <v>28</v>
+    <row r="114" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B114" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C114" s="12">
+        <v>4</v>
+      </c>
+      <c r="D114" s="24">
+        <v>46247</v>
+      </c>
+      <c r="E114" s="24">
+        <v>46266</v>
+      </c>
+      <c r="F114" s="12" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="115" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B115" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="C115" s="15">
-        <v>100</v>
-      </c>
-      <c r="D115" s="25">
-        <v>46252</v>
-      </c>
-      <c r="E115" s="25">
-        <v>46269</v>
-      </c>
-      <c r="F115" s="15" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="116" spans="2:6" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+      <c r="C115" s="12">
+        <v>6</v>
+      </c>
+      <c r="D115" s="24">
+        <v>46247</v>
+      </c>
+      <c r="E115" s="24">
+        <v>46266</v>
+      </c>
+      <c r="F115" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="116" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B116" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="C116" s="15">
-        <v>2</v>
-      </c>
-      <c r="D116" s="25">
-        <v>46252</v>
-      </c>
-      <c r="E116" s="25">
-        <v>46269</v>
-      </c>
-      <c r="F116" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="C116" s="12">
+        <v>4</v>
+      </c>
+      <c r="D116" s="24">
+        <v>46247</v>
+      </c>
+      <c r="E116" s="24">
+        <v>46266</v>
+      </c>
+      <c r="F116" s="12" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="117" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B117" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="C117" s="15">
-        <v>2</v>
-      </c>
-      <c r="D117" s="25">
-        <v>46252</v>
-      </c>
-      <c r="E117" s="25">
-        <v>46269</v>
-      </c>
-      <c r="F117" s="15" t="s">
-        <v>25</v>
+      <c r="B117" s="35" t="s">
+        <v>66</v>
+      </c>
+      <c r="C117" s="12">
+        <v>47</v>
+      </c>
+      <c r="D117" s="24">
+        <v>46251</v>
+      </c>
+      <c r="E117" s="24">
+        <v>46268</v>
+      </c>
+      <c r="F117" s="12" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="118" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B118" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="C118" s="15">
+        <v>20</v>
+      </c>
+      <c r="C118" s="12">
+        <v>100</v>
+      </c>
+      <c r="D118" s="24">
+        <v>46251</v>
+      </c>
+      <c r="E118" s="24">
+        <v>46269</v>
+      </c>
+      <c r="F118" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="119" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B119" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C119" s="12">
+        <v>2</v>
+      </c>
+      <c r="D119" s="24">
+        <v>46252</v>
+      </c>
+      <c r="E119" s="24">
+        <v>46270</v>
+      </c>
+      <c r="F119" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="120" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B120" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C120" s="12">
         <v>1</v>
       </c>
-      <c r="D118" s="25">
+      <c r="D120" s="24">
         <v>46252</v>
       </c>
-      <c r="E118" s="25">
-        <v>46269</v>
-      </c>
-      <c r="F118" s="15" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="119" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B119" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="C119" s="15">
-        <v>10</v>
-      </c>
-      <c r="D119" s="25">
-        <v>46258</v>
-      </c>
-      <c r="E119" s="25">
+      <c r="E120" s="24">
+        <v>46270</v>
+      </c>
+      <c r="F120" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="121" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B121" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="C121" s="12">
+        <v>2</v>
+      </c>
+      <c r="D121" s="24">
+        <v>46252</v>
+      </c>
+      <c r="E121" s="24">
+        <v>46270</v>
+      </c>
+      <c r="F121" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="122" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B122" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C122" s="12">
+        <v>30</v>
+      </c>
+      <c r="D122" s="24">
+        <v>46256</v>
+      </c>
+      <c r="E122" s="24">
         <v>46273</v>
       </c>
-      <c r="F119" s="15" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="120" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B120" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="C120" s="15">
-        <v>13</v>
-      </c>
-      <c r="D120" s="25">
-        <v>46261</v>
-      </c>
-      <c r="E120" s="25">
-        <v>46277</v>
-      </c>
-      <c r="F120" s="15" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="121" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B121" s="35" t="s">
-        <v>70</v>
-      </c>
-      <c r="C121" s="15">
-        <v>13</v>
-      </c>
-      <c r="D121" s="25">
+      <c r="F122" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="123" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B123" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C123" s="12">
+        <v>4</v>
+      </c>
+      <c r="D123" s="24">
         <v>46256</v>
       </c>
-      <c r="F121" s="15" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="122" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B122" s="35" t="s">
-        <v>70</v>
-      </c>
-      <c r="C122" s="15">
-        <v>60</v>
-      </c>
-      <c r="D122" s="25">
-        <v>46255</v>
-      </c>
-      <c r="F122" s="15" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="123" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B123" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="C123" s="15">
-        <v>36</v>
-      </c>
-      <c r="D123" s="25">
-        <v>46256</v>
-      </c>
-      <c r="F123" s="15" t="s">
+      <c r="E123" s="24">
+        <v>46273</v>
+      </c>
+      <c r="F123" s="12" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="124" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B124" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C124" s="12">
         <v>8</v>
@@ -2961,7 +2955,7 @@
     </row>
     <row r="125" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B125" s="12" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C125" s="12">
         <v>10</v>
@@ -2977,8 +2971,8 @@
       </c>
     </row>
     <row r="126" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B126" s="15" t="s">
-        <v>35</v>
+      <c r="B126" s="12" t="s">
+        <v>31</v>
       </c>
       <c r="C126" s="12">
         <v>1</v>
@@ -2994,8 +2988,8 @@
       </c>
     </row>
     <row r="127" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B127" s="12" t="s">
-        <v>73</v>
+      <c r="B127" s="15" t="s">
+        <v>70</v>
       </c>
       <c r="C127" s="12">
         <v>1</v>
@@ -3012,7 +3006,7 @@
     </row>
     <row r="128" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B128" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C128" s="12">
         <v>58</v>
@@ -3029,7 +3023,7 @@
     </row>
     <row r="129" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B129" s="12" t="s">
-        <v>74</v>
+        <v>22</v>
       </c>
       <c r="C129" s="12">
         <v>47</v>
@@ -3046,7 +3040,7 @@
     </row>
     <row r="130" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B130" s="12" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C130" s="12">
         <v>10</v>
@@ -3080,7 +3074,7 @@
     </row>
     <row r="132" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B132" s="12" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="C132" s="12">
         <v>6</v>
@@ -3096,8 +3090,8 @@
       </c>
     </row>
     <row r="133" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B133" s="12" t="s">
-        <v>76</v>
+      <c r="B133" s="9" t="s">
+        <v>23</v>
       </c>
       <c r="C133" s="12">
         <v>10</v>
@@ -3114,7 +3108,7 @@
     </row>
     <row r="134" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B134" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C134" s="12">
         <v>29</v>
@@ -3130,8 +3124,8 @@
       </c>
     </row>
     <row r="135" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B135" s="12" t="s">
-        <v>77</v>
+      <c r="B135" s="15" t="s">
+        <v>34</v>
       </c>
       <c r="C135" s="12">
         <v>1</v>
@@ -3148,7 +3142,7 @@
     </row>
     <row r="136" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B136" s="35" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C136" s="15">
         <v>48</v>
@@ -3160,15 +3154,14 @@
         <v>46281</v>
       </c>
       <c r="F136" s="15" t="s">
-        <v>29</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="B1:E136" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="0">
       <filters>
-        <filter val="APPRENTIS MOTNAGE"/>
-        <filter val="Montage apprentis"/>
+        <filter val="MOT APRRENTIS"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -3187,7 +3180,7 @@
   <sheetData>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="36" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B4" s="36"/>
       <c r="C4" s="36"/>
@@ -3284,7 +3277,7 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -3412,7 +3405,7 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B1" t="s">
         <v>2</v>
@@ -3450,7 +3443,7 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B2">
         <v>100</v>
@@ -3488,7 +3481,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B3">
         <v>70</v>
@@ -3526,7 +3519,7 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B4">
         <v>20</v>
@@ -3564,7 +3557,7 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D5">
         <v>950</v>
@@ -3578,7 +3571,7 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D6">
         <v>305</v>
@@ -3592,7 +3585,7 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E7">
         <v>30</v>
@@ -3603,7 +3596,7 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="F8">
         <v>330</v>
@@ -3621,47 +3614,47 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" t="s">
         <v>45</v>
-      </c>
-      <c r="B1" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" t="s">
         <v>47</v>
-      </c>
-      <c r="B2" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" t="s">
         <v>49</v>
-      </c>
-      <c r="B3" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" t="s">
         <v>51</v>
-      </c>
-      <c r="B4" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" t="s">
         <v>53</v>
-      </c>
-      <c r="B5" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B6">
         <v>50</v>
@@ -3669,7 +3662,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B7">
         <v>30</v>
@@ -3690,13 +3683,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1" t="s">
         <v>57</v>
       </c>
-      <c r="B1" t="s">
-        <v>58</v>
-      </c>
       <c r="C1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -3704,7 +3697,7 @@
         <v>46245</v>
       </c>
       <c r="B2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C2">
         <v>141</v>
@@ -3715,7 +3708,7 @@
         <v>46246</v>
       </c>
       <c r="B3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C3">
         <v>66</v>
@@ -3726,7 +3719,7 @@
         <v>46247</v>
       </c>
       <c r="B4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C4">
         <v>67</v>
@@ -3747,10 +3740,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1" t="s">
         <v>61</v>
-      </c>
-      <c r="B1" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -3763,7 +3756,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B3">
         <v>46</v>
@@ -3787,7 +3780,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B6">
         <v>6</v>
@@ -3795,7 +3788,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B7">
         <v>4</v>
@@ -3803,7 +3796,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B8">
         <v>4</v>

</xml_diff>

<commit_message>
update the excel values
</commit_message>
<xml_diff>
--- a/suivi.xlsx
+++ b/suivi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\user\TA38804\Documents\ALL PFE Projects\dashboard-static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C269CE5B-3051-42C2-B2EC-514DE0D4D1D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F86F6F7F-CF5F-4239-881B-5D0F1189AFFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="74">
   <si>
     <t>Des arrivees Non diplomes</t>
   </si>
@@ -261,6 +261,9 @@
   </si>
   <si>
     <t>NOn</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> MOT</t>
   </si>
 </sst>
 </file>
@@ -899,8 +902,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="B1:F136"/>
+  <dimension ref="B1:F147"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="15" customWidth="1"/>
@@ -926,7 +928,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
         <v>19</v>
       </c>
@@ -941,7 +943,7 @@
       </c>
       <c r="F2" s="16"/>
     </row>
-    <row r="3" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="35" t="s">
         <v>66</v>
       </c>
@@ -956,7 +958,7 @@
       </c>
       <c r="F3" s="16"/>
     </row>
-    <row r="4" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="15" t="s">
         <v>20</v>
       </c>
@@ -971,7 +973,7 @@
       </c>
       <c r="F4" s="16"/>
     </row>
-    <row r="5" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="s">
         <v>21</v>
       </c>
@@ -986,7 +988,7 @@
       </c>
       <c r="F5" s="16"/>
     </row>
-    <row r="6" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="35" t="s">
         <v>66</v>
       </c>
@@ -1001,7 +1003,7 @@
       </c>
       <c r="F6" s="16"/>
     </row>
-    <row r="7" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="15" t="s">
         <v>20</v>
       </c>
@@ -1016,7 +1018,7 @@
       </c>
       <c r="F7" s="16"/>
     </row>
-    <row r="8" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
         <v>22</v>
       </c>
@@ -1031,7 +1033,7 @@
       </c>
       <c r="F8" s="16"/>
     </row>
-    <row r="9" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
         <v>19</v>
       </c>
@@ -1046,7 +1048,7 @@
       </c>
       <c r="F9" s="16"/>
     </row>
-    <row r="10" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
         <v>22</v>
       </c>
@@ -1061,7 +1063,7 @@
       </c>
       <c r="F10" s="16"/>
     </row>
-    <row r="11" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="3" t="s">
         <v>21</v>
       </c>
@@ -1076,7 +1078,7 @@
       </c>
       <c r="F11" s="16"/>
     </row>
-    <row r="12" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="35" t="s">
         <v>66</v>
       </c>
@@ -1091,7 +1093,7 @@
       </c>
       <c r="F12" s="16"/>
     </row>
-    <row r="13" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
         <v>23</v>
       </c>
@@ -1106,7 +1108,7 @@
       </c>
       <c r="F13" s="16"/>
     </row>
-    <row r="14" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="15" t="s">
         <v>20</v>
       </c>
@@ -1121,7 +1123,7 @@
       </c>
       <c r="F14" s="16"/>
     </row>
-    <row r="15" spans="2:6" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
         <v>19</v>
       </c>
@@ -1136,7 +1138,7 @@
       </c>
       <c r="F15" s="16"/>
     </row>
-    <row r="16" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16" s="35" t="s">
         <v>66</v>
       </c>
@@ -1150,7 +1152,7 @@
         <v>46177</v>
       </c>
     </row>
-    <row r="17" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="15" t="s">
         <v>20</v>
       </c>
@@ -1164,7 +1166,7 @@
         <v>46177</v>
       </c>
     </row>
-    <row r="18" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
         <v>23</v>
       </c>
@@ -1178,7 +1180,7 @@
         <v>46177</v>
       </c>
     </row>
-    <row r="19" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19" s="4" t="s">
         <v>19</v>
       </c>
@@ -1192,7 +1194,7 @@
         <v>46177</v>
       </c>
     </row>
-    <row r="20" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" s="35" t="s">
         <v>66</v>
       </c>
@@ -1206,7 +1208,7 @@
         <v>46177</v>
       </c>
     </row>
-    <row r="21" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" s="4" t="s">
         <v>21</v>
       </c>
@@ -1220,7 +1222,7 @@
         <v>46178</v>
       </c>
     </row>
-    <row r="22" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" s="35" t="s">
         <v>66</v>
       </c>
@@ -1234,7 +1236,7 @@
         <v>46183</v>
       </c>
     </row>
-    <row r="23" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" s="15" t="s">
         <v>20</v>
       </c>
@@ -1248,7 +1250,7 @@
         <v>46183</v>
       </c>
     </row>
-    <row r="24" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" s="5" t="s">
         <v>23</v>
       </c>
@@ -1262,7 +1264,7 @@
         <v>46183</v>
       </c>
     </row>
-    <row r="25" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" s="5" t="s">
         <v>19</v>
       </c>
@@ -1276,7 +1278,7 @@
         <v>46183</v>
       </c>
     </row>
-    <row r="26" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" s="5" t="s">
         <v>24</v>
       </c>
@@ -1290,7 +1292,7 @@
         <v>46183</v>
       </c>
     </row>
-    <row r="27" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" s="35" t="s">
         <v>66</v>
       </c>
@@ -1304,7 +1306,7 @@
         <v>46184</v>
       </c>
     </row>
-    <row r="28" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28" s="15" t="s">
         <v>20</v>
       </c>
@@ -1321,7 +1323,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B29" s="35" t="s">
         <v>66</v>
       </c>
@@ -1338,7 +1340,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30" s="6" t="s">
         <v>19</v>
       </c>
@@ -1355,7 +1357,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="31" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B31" s="6" t="s">
         <v>21</v>
       </c>
@@ -1372,7 +1374,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B32" s="6" t="s">
         <v>23</v>
       </c>
@@ -1389,7 +1391,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="33" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B33" s="35" t="s">
         <v>66</v>
       </c>
@@ -1406,7 +1408,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B34" s="7" t="s">
         <v>23</v>
       </c>
@@ -1423,7 +1425,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B35" s="7" t="s">
         <v>24</v>
       </c>
@@ -1440,7 +1442,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="36" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B36" s="7" t="s">
         <v>22</v>
       </c>
@@ -1457,7 +1459,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="37" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B37" s="7" t="s">
         <v>19</v>
       </c>
@@ -1474,7 +1476,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="38" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B38" s="7" t="s">
         <v>23</v>
       </c>
@@ -1491,7 +1493,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="39" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B39" s="35" t="s">
         <v>66</v>
       </c>
@@ -1508,7 +1510,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="40" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B40" s="15" t="s">
         <v>20</v>
       </c>
@@ -1525,7 +1527,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="41" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B41" s="7" t="s">
         <v>19</v>
       </c>
@@ -1542,7 +1544,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="42" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B42" s="15" t="s">
         <v>20</v>
       </c>
@@ -1559,7 +1561,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="43" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B43" s="7" t="s">
         <v>22</v>
       </c>
@@ -1576,7 +1578,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="44" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B44" s="7" t="s">
         <v>21</v>
       </c>
@@ -1593,7 +1595,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="45" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B45" s="7" t="s">
         <v>21</v>
       </c>
@@ -1610,7 +1612,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="46" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B46" s="7" t="s">
         <v>26</v>
       </c>
@@ -1627,7 +1629,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="47" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B47" s="7" t="s">
         <v>27</v>
       </c>
@@ -1644,7 +1646,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="48" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B48" s="35" t="s">
         <v>66</v>
       </c>
@@ -1661,7 +1663,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="49" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B49" s="35" t="s">
         <v>66</v>
       </c>
@@ -1678,7 +1680,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="50" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B50" s="35" t="s">
         <v>66</v>
       </c>
@@ -1695,7 +1697,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="51" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B51" s="35" t="s">
         <v>66</v>
       </c>
@@ -1712,7 +1714,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="52" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B52" s="35" t="s">
         <v>66</v>
       </c>
@@ -1729,7 +1731,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="53" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B53" s="35" t="s">
         <v>66</v>
       </c>
@@ -1746,7 +1748,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="54" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B54" s="35" t="s">
         <v>66</v>
       </c>
@@ -1763,7 +1765,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="55" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B55" s="15" t="s">
         <v>20</v>
       </c>
@@ -1780,7 +1782,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="56" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B56" s="15" t="s">
         <v>20</v>
       </c>
@@ -1797,7 +1799,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="57" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B57" s="9" t="s">
         <v>26</v>
       </c>
@@ -1814,7 +1816,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="58" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B58" s="9" t="s">
         <v>23</v>
       </c>
@@ -1831,7 +1833,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="59" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B59" s="9" t="s">
         <v>23</v>
       </c>
@@ -1848,7 +1850,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="60" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B60" s="9" t="s">
         <v>22</v>
       </c>
@@ -1865,7 +1867,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="61" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B61" s="9" t="s">
         <v>19</v>
       </c>
@@ -1882,7 +1884,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="62" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B62" s="9" t="s">
         <v>19</v>
       </c>
@@ -1899,7 +1901,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="63" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B63" s="9" t="s">
         <v>21</v>
       </c>
@@ -1916,7 +1918,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="64" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B64" s="9" t="s">
         <v>23</v>
       </c>
@@ -1933,7 +1935,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="65" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B65" s="35" t="s">
         <v>66</v>
       </c>
@@ -1950,7 +1952,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="66" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B66" s="35" t="s">
         <v>66</v>
       </c>
@@ -1967,7 +1969,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="67" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B67" s="9" t="s">
         <v>21</v>
       </c>
@@ -1984,7 +1986,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="68" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B68" s="35" t="s">
         <v>66</v>
       </c>
@@ -2001,7 +2003,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="69" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B69" s="9" t="s">
         <v>19</v>
       </c>
@@ -2018,7 +2020,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="70" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B70" s="9" t="s">
         <v>23</v>
       </c>
@@ -2035,7 +2037,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="71" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B71" s="9" t="s">
         <v>26</v>
       </c>
@@ -2052,7 +2054,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="72" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B72" s="9" t="s">
         <v>23</v>
       </c>
@@ -2069,7 +2071,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="73" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B73" s="15" t="s">
         <v>20</v>
       </c>
@@ -2086,7 +2088,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="74" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B74" s="9" t="s">
         <v>21</v>
       </c>
@@ -2103,7 +2105,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="75" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B75" s="35" t="s">
         <v>66</v>
       </c>
@@ -2120,7 +2122,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="76" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B76" s="35" t="s">
         <v>66</v>
       </c>
@@ -2137,7 +2139,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="77" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B77" s="35" t="s">
         <v>66</v>
       </c>
@@ -2154,7 +2156,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="78" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B78" s="9" t="s">
         <v>23</v>
       </c>
@@ -2171,7 +2173,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="79" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B79" s="35" t="s">
         <v>66</v>
       </c>
@@ -2188,7 +2190,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="80" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B80" s="35" t="s">
         <v>66</v>
       </c>
@@ -2205,7 +2207,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="81" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B81" s="9" t="s">
         <v>27</v>
       </c>
@@ -2222,7 +2224,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="82" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B82" s="15" t="s">
         <v>20</v>
       </c>
@@ -2239,7 +2241,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="83" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B83" s="9" t="s">
         <v>23</v>
       </c>
@@ -2256,7 +2258,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="84" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B84" s="35" t="s">
         <v>66</v>
       </c>
@@ -2273,7 +2275,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="85" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B85" s="12" t="s">
         <v>22</v>
       </c>
@@ -2290,7 +2292,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="86" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B86" s="15" t="s">
         <v>20</v>
       </c>
@@ -2307,7 +2309,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="87" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B87" s="35" t="s">
         <v>66</v>
       </c>
@@ -2324,7 +2326,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="88" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B88" s="35" t="s">
         <v>66</v>
       </c>
@@ -2341,7 +2343,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="89" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B89" s="15" t="s">
         <v>20</v>
       </c>
@@ -2358,7 +2360,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="90" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B90" s="14" t="s">
         <v>30</v>
       </c>
@@ -2375,7 +2377,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="91" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B91" s="12" t="s">
         <v>21</v>
       </c>
@@ -2392,7 +2394,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="92" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B92" s="35" t="s">
         <v>66</v>
       </c>
@@ -2409,7 +2411,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="93" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B93" s="12" t="s">
         <v>21</v>
       </c>
@@ -2426,7 +2428,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="94" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B94" s="15" t="s">
         <v>20</v>
       </c>
@@ -2443,7 +2445,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="95" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B95" s="35" t="s">
         <v>66</v>
       </c>
@@ -2477,7 +2479,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="97" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B97" s="12" t="s">
         <v>32</v>
       </c>
@@ -2494,7 +2496,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="98" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B98" s="12" t="s">
         <v>24</v>
       </c>
@@ -2511,7 +2513,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="99" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B99" s="12" t="s">
         <v>32</v>
       </c>
@@ -2528,7 +2530,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="100" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B100" s="35" t="s">
         <v>66</v>
       </c>
@@ -2545,7 +2547,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="101" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B101" s="15" t="s">
         <v>20</v>
       </c>
@@ -2562,7 +2564,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="102" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B102" s="9" t="s">
         <v>23</v>
       </c>
@@ -2579,7 +2581,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="103" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B103" s="12" t="s">
         <v>32</v>
       </c>
@@ -2596,7 +2598,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="104" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B104" s="12" t="s">
         <v>33</v>
       </c>
@@ -2613,7 +2615,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="105" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B105" s="35" t="s">
         <v>66</v>
       </c>
@@ -2630,7 +2632,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="106" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B106" s="35" t="s">
         <v>66</v>
       </c>
@@ -2647,7 +2649,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="107" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B107" s="35" t="s">
         <v>66</v>
       </c>
@@ -2664,7 +2666,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="108" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B108" s="15" t="s">
         <v>20</v>
       </c>
@@ -2681,7 +2683,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="109" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B109" s="15" t="s">
         <v>21</v>
       </c>
@@ -2698,7 +2700,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="110" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B110" s="12" t="s">
         <v>32</v>
       </c>
@@ -2715,7 +2717,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="111" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B111" s="15" t="s">
         <v>34</v>
       </c>
@@ -2749,7 +2751,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="113" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B113" s="15" t="s">
         <v>70</v>
       </c>
@@ -2783,7 +2785,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="115" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B115" s="15" t="s">
         <v>34</v>
       </c>
@@ -2800,7 +2802,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="116" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B116" s="15" t="s">
         <v>70</v>
       </c>
@@ -2817,7 +2819,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="117" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B117" s="35" t="s">
         <v>66</v>
       </c>
@@ -2834,7 +2836,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="118" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B118" s="15" t="s">
         <v>20</v>
       </c>
@@ -2868,7 +2870,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="120" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B120" s="12" t="s">
         <v>33</v>
       </c>
@@ -2885,7 +2887,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="121" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B121" s="12" t="s">
         <v>71</v>
       </c>
@@ -2902,7 +2904,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="122" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B122" s="15" t="s">
         <v>20</v>
       </c>
@@ -2919,7 +2921,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="123" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B123" s="9" t="s">
         <v>23</v>
       </c>
@@ -2936,7 +2938,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="124" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B124" s="35" t="s">
         <v>66</v>
       </c>
@@ -2953,7 +2955,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="125" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B125" s="12" t="s">
         <v>68</v>
       </c>
@@ -2987,7 +2989,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="127" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B127" s="15" t="s">
         <v>70</v>
       </c>
@@ -3004,7 +3006,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="128" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B128" s="35" t="s">
         <v>66</v>
       </c>
@@ -3021,7 +3023,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="129" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B129" s="12" t="s">
         <v>22</v>
       </c>
@@ -3038,7 +3040,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="130" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B130" s="12" t="s">
         <v>68</v>
       </c>
@@ -3055,7 +3057,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="131" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B131" s="15" t="s">
         <v>20</v>
       </c>
@@ -3072,7 +3074,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="132" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B132" s="12" t="s">
         <v>69</v>
       </c>
@@ -3089,7 +3091,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="133" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B133" s="9" t="s">
         <v>23</v>
       </c>
@@ -3106,7 +3108,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="134" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B134" s="35" t="s">
         <v>66</v>
       </c>
@@ -3123,7 +3125,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="135" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B135" s="15" t="s">
         <v>34</v>
       </c>
@@ -3140,7 +3142,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="136" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B136" s="35" t="s">
         <v>66</v>
       </c>
@@ -3157,14 +3159,86 @@
         <v>72</v>
       </c>
     </row>
+    <row r="137" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B137" s="35" t="s">
+        <v>66</v>
+      </c>
+      <c r="C137" s="15">
+        <v>62</v>
+      </c>
+      <c r="D137" s="25">
+        <v>46268</v>
+      </c>
+      <c r="F137" s="15" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="138" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B138" s="35" t="s">
+        <v>66</v>
+      </c>
+      <c r="C138" s="15">
+        <v>23</v>
+      </c>
+      <c r="D138" s="25">
+        <v>46268</v>
+      </c>
+      <c r="F138" s="15" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="139" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B139" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C139" s="15">
+        <v>40</v>
+      </c>
+      <c r="D139" s="25">
+        <v>46268</v>
+      </c>
+    </row>
+    <row r="140" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B140" t="s">
+        <v>20</v>
+      </c>
+      <c r="C140" s="15">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="141" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B141" t="s">
+        <v>19</v>
+      </c>
+      <c r="C141" s="15">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="142" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B142" t="s">
+        <v>73</v>
+      </c>
+      <c r="C142" s="15">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="143" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B143"/>
+    </row>
+    <row r="144" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B144"/>
+    </row>
+    <row r="145" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B145"/>
+    </row>
+    <row r="146" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B146"/>
+    </row>
+    <row r="147" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B147"/>
+    </row>
   </sheetData>
-  <autoFilter ref="B1:E136" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="MOT APRRENTIS"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="B1:E136" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>